<commit_message>
updated silicon mass baseline
again, should weight by tech, did by eyeballing p-type v n-type
</commit_message>
<xml_diff>
--- a/PV_ICE/baselines/SupportingMaterial/Manual Files/BaselineGraphs.xlsx
+++ b/PV_ICE/baselines/SupportingMaterial/Manual Files/BaselineGraphs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmirletz\Documents\GitHub\PV_ICE\PV_ICE\baselines\SupportingMaterial\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmirletz\Documents\GitHub\PV_ICE\PV_ICE\baselines\SupportingMaterial\Manual Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BA104A-C648-4039-9CC4-A304B7711A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A77E539-5F2C-4B89-87CA-73FC844C1CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2865" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{31D47E9D-A833-4D35-B79A-EFF0E4DE6D01}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{31D47E9D-A833-4D35-B79A-EFF0E4DE6D01}"/>
   </bookViews>
   <sheets>
     <sheet name="mass per m2" sheetId="1" r:id="rId1"/>
@@ -235,16 +235,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -955,6 +949,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -962,7 +957,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3964,6 +3958,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3971,7 +3966,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6975,6 +6969,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6982,7 +6977,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7604,6 +7598,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7611,7 +7606,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8561,6 +8555,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8568,7 +8563,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9518,6 +9512,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9525,7 +9520,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11346,6 +11340,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11353,7 +11348,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13125,6 +13119,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13132,7 +13127,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15125,6 +15119,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15132,7 +15127,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16250,6 +16244,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -16257,7 +16252,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -17373,6 +17367,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -17380,7 +17375,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -18398,6 +18392,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -18405,7 +18400,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -19023,6 +19017,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -19030,7 +19025,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -20552,6 +20546,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -20559,7 +20554,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -22689,6 +22683,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -22696,7 +22691,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -23128,6 +23122,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -23135,7 +23130,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -28353,6 +28347,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -28360,7 +28355,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -38495,9 +38489,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -38535,7 +38529,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -38641,7 +38635,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -38783,7 +38777,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -38803,55 +38797,55 @@
     <col min="8" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.81640625" customWidth="1"/>
     <col min="10" max="10" width="7.6328125" customWidth="1"/>
-    <col min="11" max="11" width="2.453125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="2.453125" style="6" customWidth="1"/>
     <col min="12" max="13" width="8.26953125" customWidth="1"/>
     <col min="14" max="20" width="11.81640625" customWidth="1"/>
-    <col min="21" max="21" width="2.26953125" style="8" customWidth="1"/>
+    <col min="21" max="21" width="2.26953125" style="6" customWidth="1"/>
     <col min="34" max="34" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.35">
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
       <c r="I1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="3"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="6" t="s">
+      <c r="J1" s="2"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="10" t="s">
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="10"/>
-      <c r="Z1" s="10"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
       <c r="AA1" s="2"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="2"/>
-      <c r="AD1" s="10" t="s">
+      <c r="AD1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="AE1" s="10"/>
-      <c r="AF1" s="10"/>
-      <c r="AG1" s="10"/>
-      <c r="AH1" s="10"/>
+      <c r="AE1" s="8"/>
+      <c r="AF1" s="8"/>
+      <c r="AG1" s="8"/>
+      <c r="AH1" s="8"/>
       <c r="AI1" s="1" t="s">
         <v>18</v>
       </c>
@@ -39108,47 +39102,47 @@
       <c r="H18">
         <v>532</v>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="3">
         <f>SUM(B18:H18)</f>
         <v>13410.982838600001</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="3">
         <f>AD18*1000/100</f>
         <v>125</v>
       </c>
-      <c r="K18" s="9"/>
-      <c r="L18" s="5">
+      <c r="K18" s="7"/>
+      <c r="L18" s="3">
         <f>I18/J18</f>
         <v>107.28786270880001</v>
       </c>
-      <c r="M18" s="5">
+      <c r="M18" s="3">
         <v>121.9734352</v>
       </c>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="5"/>
-      <c r="R18" s="5"/>
-      <c r="S18" s="5"/>
-      <c r="T18" s="5"/>
-      <c r="U18" s="9"/>
-      <c r="V18" s="5">
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="7"/>
+      <c r="V18" s="3">
         <f t="shared" ref="V18:V49" si="0">B18/$I18*100</f>
         <v>59.652600381935436</v>
       </c>
-      <c r="W18" s="5">
+      <c r="W18" s="3">
         <f t="shared" ref="W18:W49" si="1">C18/$I18*100</f>
         <v>6.326318054468322</v>
       </c>
-      <c r="X18" s="5">
+      <c r="X18" s="3">
         <f t="shared" ref="X18:X49" si="2">D18/$I18*100</f>
         <v>23.049655996149905</v>
       </c>
-      <c r="Y18" s="5">
+      <c r="Y18" s="3">
         <f t="shared" ref="Y18:Y49" si="3">E18/$I18*100</f>
         <v>4.0086547456660612E-2</v>
       </c>
-      <c r="Z18" s="5">
+      <c r="Z18" s="3">
         <f t="shared" ref="Z18:Z49" si="4">F18/$I18*100</f>
         <v>0.65617860420128982</v>
       </c>
@@ -39193,47 +39187,47 @@
       <c r="H19">
         <v>532</v>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="3">
         <f t="shared" ref="I19:I73" si="5">SUM(B19:H19)</f>
         <v>13317.14968887</v>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="3">
         <f t="shared" ref="J19:J73" si="6">AD19*1000/100</f>
         <v>127</v>
       </c>
-      <c r="K19" s="9"/>
-      <c r="L19" s="5">
+      <c r="K19" s="7"/>
+      <c r="L19" s="3">
         <f t="shared" ref="L19:L73" si="7">I19/J19</f>
         <v>104.85944636905512</v>
       </c>
-      <c r="M19" s="5">
+      <c r="M19" s="3">
         <v>119.3832118</v>
       </c>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5"/>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
-      <c r="U19" s="9"/>
-      <c r="V19" s="5">
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
+      <c r="R19" s="3"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+      <c r="U19" s="7"/>
+      <c r="V19" s="3">
         <f t="shared" si="0"/>
         <v>60.072914902249053</v>
       </c>
-      <c r="W19" s="5">
+      <c r="W19" s="3">
         <f t="shared" si="1"/>
         <v>6.2459740540062931</v>
       </c>
-      <c r="X19" s="5">
+      <c r="X19" s="3">
         <f t="shared" si="2"/>
         <v>22.658125924062034</v>
       </c>
-      <c r="Y19" s="5">
+      <c r="Y19" s="3">
         <f t="shared" si="3"/>
         <v>4.0368998814311365E-2</v>
       </c>
-      <c r="Z19" s="5">
+      <c r="Z19" s="3">
         <f t="shared" si="4"/>
         <v>0.63505652895590559</v>
       </c>
@@ -39278,47 +39272,47 @@
       <c r="H20">
         <v>532</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="3">
         <f t="shared" si="5"/>
         <v>12979.668857139999</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="3">
         <f t="shared" si="6"/>
         <v>128.80000000000001</v>
       </c>
-      <c r="K20" s="9"/>
-      <c r="L20" s="5">
+      <c r="K20" s="7"/>
+      <c r="L20" s="3">
         <f t="shared" si="7"/>
         <v>100.77382653059004</v>
       </c>
-      <c r="M20" s="5">
+      <c r="M20" s="3">
         <v>116.8479943</v>
       </c>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-      <c r="R20" s="5"/>
-      <c r="S20" s="5"/>
-      <c r="T20" s="5"/>
-      <c r="U20" s="9"/>
-      <c r="V20" s="5">
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
+      <c r="R20" s="3"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+      <c r="U20" s="7"/>
+      <c r="V20" s="3">
         <f t="shared" si="0"/>
         <v>61.634854386899654</v>
       </c>
-      <c r="W20" s="5">
+      <c r="W20" s="3">
         <f t="shared" si="1"/>
         <v>6.2802064441851559</v>
       </c>
-      <c r="X20" s="5">
+      <c r="X20" s="3">
         <f t="shared" si="2"/>
         <v>20.801763355578633</v>
       </c>
-      <c r="Y20" s="5">
+      <c r="Y20" s="3">
         <f t="shared" si="3"/>
         <v>4.1418622147996562E-2</v>
       </c>
-      <c r="Z20" s="5">
+      <c r="Z20" s="3">
         <f t="shared" si="4"/>
         <v>0.62515352304511262</v>
       </c>
@@ -39363,47 +39357,47 @@
       <c r="H21">
         <v>532</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="3">
         <f t="shared" si="5"/>
         <v>12799.977242410001</v>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="3">
         <f t="shared" si="6"/>
         <v>130.6</v>
       </c>
-      <c r="K21" s="9"/>
-      <c r="L21" s="5">
+      <c r="K21" s="7"/>
+      <c r="L21" s="3">
         <f t="shared" si="7"/>
         <v>98.009014107274126</v>
       </c>
-      <c r="M21" s="5">
+      <c r="M21" s="3">
         <v>114.36661460000001</v>
       </c>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-      <c r="R21" s="5"/>
-      <c r="S21" s="5"/>
-      <c r="T21" s="5"/>
-      <c r="U21" s="9"/>
-      <c r="V21" s="5">
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+      <c r="U21" s="7"/>
+      <c r="V21" s="3">
         <f t="shared" si="0"/>
         <v>62.500111121242483</v>
       </c>
-      <c r="W21" s="5">
+      <c r="W21" s="3">
         <f t="shared" si="1"/>
         <v>6.2384039485186955</v>
       </c>
-      <c r="X21" s="5">
+      <c r="X21" s="3">
         <f t="shared" si="2"/>
         <v>19.846696778358446</v>
       </c>
-      <c r="Y21" s="5">
+      <c r="Y21" s="3">
         <f t="shared" si="3"/>
         <v>4.2000074673474955E-2</v>
       </c>
-      <c r="Z21" s="5">
+      <c r="Z21" s="3">
         <f t="shared" si="4"/>
         <v>0.60714393657287336</v>
       </c>
@@ -39448,47 +39442,47 @@
       <c r="H22">
         <v>532</v>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="3">
         <f t="shared" si="5"/>
         <v>12724.239199690001</v>
       </c>
-      <c r="J22" s="5">
+      <c r="J22" s="3">
         <f t="shared" si="6"/>
         <v>132.4</v>
       </c>
-      <c r="K22" s="9"/>
-      <c r="L22" s="5">
+      <c r="K22" s="7"/>
+      <c r="L22" s="3">
         <f t="shared" si="7"/>
         <v>96.104525677416916</v>
       </c>
-      <c r="M22" s="5">
+      <c r="M22" s="3">
         <v>111.9379294</v>
       </c>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="5"/>
-      <c r="U22" s="9"/>
-      <c r="V22" s="5">
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="3"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+      <c r="U22" s="7"/>
+      <c r="V22" s="3">
         <f t="shared" si="0"/>
         <v>62.872128340646903</v>
       </c>
-      <c r="W22" s="5">
+      <c r="W22" s="3">
         <f t="shared" si="1"/>
         <v>6.144796235982807</v>
       </c>
-      <c r="X22" s="5">
+      <c r="X22" s="3">
         <f t="shared" si="2"/>
         <v>19.52728862610925</v>
       </c>
-      <c r="Y22" s="5">
+      <c r="Y22" s="3">
         <f t="shared" si="3"/>
         <v>4.2250070244914728E-2</v>
       </c>
-      <c r="Z22" s="5">
+      <c r="Z22" s="3">
         <f t="shared" si="4"/>
         <v>0.5838126203396885</v>
       </c>
@@ -39533,49 +39527,49 @@
       <c r="H23">
         <v>532</v>
       </c>
-      <c r="I23" s="5">
+      <c r="I23" s="3">
         <f t="shared" si="5"/>
         <v>12627.92969253</v>
       </c>
-      <c r="J23" s="5">
+      <c r="J23" s="3">
         <f t="shared" si="6"/>
         <v>134.19999999999999</v>
       </c>
-      <c r="K23" s="9"/>
-      <c r="L23" s="5">
+      <c r="K23" s="7"/>
+      <c r="L23" s="3">
         <f t="shared" si="7"/>
         <v>94.097836755067078</v>
       </c>
-      <c r="M23" s="5">
+      <c r="M23" s="3">
         <v>109.5608196</v>
       </c>
-      <c r="N23" s="5">
+      <c r="N23" s="3">
         <v>110</v>
       </c>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="9"/>
-      <c r="V23" s="5">
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="7"/>
+      <c r="V23" s="3">
         <f t="shared" si="0"/>
         <v>63.351635579127176</v>
       </c>
-      <c r="W23" s="5">
+      <c r="W23" s="3">
         <f t="shared" si="1"/>
         <v>6.0599233265661612</v>
       </c>
-      <c r="X23" s="5">
+      <c r="X23" s="3">
         <f t="shared" si="2"/>
         <v>19.274436295284413</v>
       </c>
-      <c r="Y23" s="5">
+      <c r="Y23" s="3">
         <f t="shared" si="3"/>
         <v>4.2572299109173463E-2</v>
       </c>
-      <c r="Z23" s="5">
+      <c r="Z23" s="3">
         <f t="shared" si="4"/>
         <v>0.3591132714084222</v>
       </c>
@@ -39620,49 +39614,49 @@
       <c r="H24">
         <v>532</v>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="3">
         <f t="shared" si="5"/>
         <v>12562.671303610001</v>
       </c>
-      <c r="J24" s="5">
+      <c r="J24" s="3">
         <f t="shared" si="6"/>
         <v>136</v>
       </c>
-      <c r="K24" s="9"/>
-      <c r="L24" s="5">
+      <c r="K24" s="7"/>
+      <c r="L24" s="3">
         <f t="shared" si="7"/>
         <v>92.372583114779417</v>
       </c>
-      <c r="M24" s="5">
+      <c r="M24" s="3">
         <v>107.23419010000001</v>
       </c>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="5"/>
-      <c r="R24" s="5">
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S24" s="5"/>
-      <c r="T24" s="5"/>
-      <c r="U24" s="9"/>
-      <c r="V24" s="5">
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="7"/>
+      <c r="V24" s="3">
         <f t="shared" si="0"/>
         <v>63.680723682558863</v>
       </c>
-      <c r="W24" s="5">
+      <c r="W24" s="3">
         <f t="shared" si="1"/>
         <v>5.9589805767255939</v>
       </c>
-      <c r="X24" s="5">
+      <c r="X24" s="3">
         <f t="shared" si="2"/>
         <v>19.004985622078006</v>
       </c>
-      <c r="Y24" s="5">
+      <c r="Y24" s="3">
         <f t="shared" si="3"/>
         <v>4.2793446314679559E-2</v>
       </c>
-      <c r="Z24" s="5">
+      <c r="Z24" s="3">
         <f t="shared" si="4"/>
         <v>0.34351201800208858</v>
       </c>
@@ -39707,49 +39701,49 @@
       <c r="H25">
         <v>532</v>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="3">
         <f t="shared" si="5"/>
         <v>12501.194776599999</v>
       </c>
-      <c r="J25" s="5">
+      <c r="J25" s="3">
         <f t="shared" si="6"/>
         <v>137.2222222</v>
       </c>
-      <c r="K25" s="9"/>
-      <c r="L25" s="5">
+      <c r="K25" s="7"/>
+      <c r="L25" s="3">
         <f t="shared" si="7"/>
         <v>91.101824297668301</v>
       </c>
-      <c r="M25" s="5">
+      <c r="M25" s="3">
         <v>104.9569687</v>
       </c>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="5"/>
-      <c r="R25" s="5">
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S25" s="5"/>
-      <c r="T25" s="5"/>
-      <c r="U25" s="9"/>
-      <c r="V25" s="5">
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="7"/>
+      <c r="V25" s="3">
         <f t="shared" si="0"/>
         <v>63.993883328452483</v>
       </c>
-      <c r="W25" s="5">
+      <c r="W25" s="3">
         <f t="shared" si="1"/>
         <v>5.8552117751986357</v>
       </c>
-      <c r="X25" s="5">
+      <c r="X25" s="3">
         <f t="shared" si="2"/>
         <v>18.757305920784546</v>
       </c>
-      <c r="Y25" s="5">
+      <c r="Y25" s="3">
         <f t="shared" si="3"/>
         <v>4.3003889596720073E-2</v>
       </c>
-      <c r="Z25" s="5">
+      <c r="Z25" s="3">
         <f t="shared" si="4"/>
         <v>0.32764868264167674</v>
       </c>
@@ -39794,51 +39788,51 @@
       <c r="H26">
         <v>532</v>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="3">
         <f t="shared" si="5"/>
         <v>12455.36948159</v>
       </c>
-      <c r="J26" s="5">
+      <c r="J26" s="3">
         <f t="shared" si="6"/>
         <v>138.44444439999998</v>
       </c>
-      <c r="K26" s="9"/>
-      <c r="L26" s="5">
+      <c r="K26" s="7"/>
+      <c r="L26" s="3">
         <f t="shared" si="7"/>
         <v>89.966553266690724</v>
       </c>
-      <c r="M26" s="5">
+      <c r="M26" s="3">
         <v>102.7281064</v>
       </c>
-      <c r="N26" s="5"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
-      <c r="Q26" s="5"/>
-      <c r="R26" s="5">
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S26" s="5">
+      <c r="S26" s="3">
         <v>102.7</v>
       </c>
-      <c r="T26" s="5"/>
-      <c r="U26" s="9"/>
-      <c r="V26" s="5">
+      <c r="T26" s="3"/>
+      <c r="U26" s="7"/>
+      <c r="V26" s="3">
         <f t="shared" si="0"/>
         <v>64.229327053080354</v>
       </c>
-      <c r="W26" s="5">
+      <c r="W26" s="3">
         <f t="shared" si="1"/>
         <v>5.7431914433154425</v>
       </c>
-      <c r="X26" s="5">
+      <c r="X26" s="3">
         <f t="shared" si="2"/>
         <v>18.609580843234109</v>
       </c>
-      <c r="Y26" s="5">
+      <c r="Y26" s="3">
         <f t="shared" si="3"/>
         <v>4.316210777967E-2</v>
       </c>
-      <c r="Z26" s="5">
+      <c r="Z26" s="3">
         <f t="shared" si="4"/>
         <v>0.31123696769733511</v>
       </c>
@@ -39883,51 +39877,51 @@
       <c r="H27">
         <v>532</v>
       </c>
-      <c r="I27" s="5">
+      <c r="I27" s="3">
         <f t="shared" si="5"/>
         <v>12374.66669057</v>
       </c>
-      <c r="J27" s="5">
+      <c r="J27" s="3">
         <f t="shared" si="6"/>
         <v>139.66666670000001</v>
       </c>
-      <c r="K27" s="9"/>
-      <c r="L27" s="5">
+      <c r="K27" s="7"/>
+      <c r="L27" s="3">
         <f t="shared" si="7"/>
         <v>88.601432130906574</v>
       </c>
-      <c r="M27" s="5">
+      <c r="M27" s="3">
         <v>100.5465761</v>
       </c>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="5"/>
-      <c r="Q27" s="5"/>
-      <c r="R27" s="5">
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S27" s="5">
+      <c r="S27" s="3">
         <v>102.7</v>
       </c>
-      <c r="T27" s="5"/>
-      <c r="U27" s="9"/>
-      <c r="V27" s="5">
+      <c r="T27" s="3"/>
+      <c r="U27" s="7"/>
+      <c r="V27" s="3">
         <f t="shared" si="0"/>
         <v>64.648205887406448</v>
       </c>
-      <c r="W27" s="5">
+      <c r="W27" s="3">
         <f t="shared" si="1"/>
         <v>5.6462126816913614</v>
       </c>
-      <c r="X27" s="5">
+      <c r="X27" s="3">
         <f t="shared" si="2"/>
         <v>18.230949716966343</v>
       </c>
-      <c r="Y27" s="5">
+      <c r="Y27" s="3">
         <f t="shared" si="3"/>
         <v>4.3443594356337135E-2</v>
       </c>
-      <c r="Z27" s="5">
+      <c r="Z27" s="3">
         <f t="shared" si="4"/>
         <v>0.2955346554737423</v>
       </c>
@@ -39972,55 +39966,55 @@
       <c r="H28">
         <v>532</v>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="3">
         <f t="shared" si="5"/>
         <v>12113.835995859999</v>
       </c>
-      <c r="J28" s="5">
+      <c r="J28" s="3">
         <f t="shared" si="6"/>
         <v>140.88888890000001</v>
       </c>
-      <c r="K28" s="9"/>
-      <c r="L28" s="5">
+      <c r="K28" s="7"/>
+      <c r="L28" s="3">
         <f t="shared" si="7"/>
         <v>85.981485768250664</v>
       </c>
-      <c r="M28" s="5">
+      <c r="M28" s="3">
         <v>98.411372709999995</v>
       </c>
-      <c r="N28" s="5">
+      <c r="N28" s="3">
         <v>98</v>
       </c>
-      <c r="O28" s="5"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5">
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3">
         <v>101.6</v>
       </c>
-      <c r="R28" s="5">
+      <c r="R28" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S28" s="5">
+      <c r="S28" s="3">
         <v>102.7</v>
       </c>
-      <c r="T28" s="5"/>
-      <c r="U28" s="9"/>
-      <c r="V28" s="5">
+      <c r="T28" s="3"/>
+      <c r="U28" s="7"/>
+      <c r="V28" s="3">
         <f t="shared" si="0"/>
         <v>66.040187457829745</v>
       </c>
-      <c r="W28" s="5">
+      <c r="W28" s="3">
         <f t="shared" si="1"/>
         <v>4.8064873934151713</v>
       </c>
-      <c r="X28" s="5">
+      <c r="X28" s="3">
         <f t="shared" si="2"/>
         <v>17.449739733329881</v>
       </c>
-      <c r="Y28" s="5">
+      <c r="Y28" s="3">
         <f t="shared" si="3"/>
         <v>4.4379005971661591E-2</v>
       </c>
-      <c r="Z28" s="5">
+      <c r="Z28" s="3">
         <f t="shared" si="4"/>
         <v>0.28378411984237417</v>
       </c>
@@ -40065,53 +40059,53 @@
       <c r="H29">
         <v>532</v>
       </c>
-      <c r="I29" s="5">
+      <c r="I29" s="3">
         <f t="shared" si="5"/>
         <v>11964.83833814</v>
       </c>
-      <c r="J29" s="5">
+      <c r="J29" s="3">
         <f t="shared" si="6"/>
         <v>142.11111109999999</v>
       </c>
-      <c r="K29" s="9"/>
-      <c r="L29" s="5">
+      <c r="K29" s="7"/>
+      <c r="L29" s="3">
         <f t="shared" si="7"/>
         <v>84.193545779264554</v>
       </c>
-      <c r="M29" s="5">
+      <c r="M29" s="3">
         <v>96.321512409999997</v>
       </c>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
-      <c r="Q29" s="5">
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3">
         <v>101.6</v>
       </c>
-      <c r="R29" s="5">
+      <c r="R29" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S29" s="5">
+      <c r="S29" s="3">
         <v>102.7</v>
       </c>
-      <c r="T29" s="5"/>
-      <c r="U29" s="9"/>
-      <c r="V29" s="5">
+      <c r="T29" s="3"/>
+      <c r="U29" s="7"/>
+      <c r="V29" s="3">
         <f t="shared" si="0"/>
         <v>66.862583295409934</v>
       </c>
-      <c r="W29" s="5">
+      <c r="W29" s="3">
         <f t="shared" si="1"/>
         <v>3.8930739123752436</v>
       </c>
-      <c r="X29" s="5">
+      <c r="X29" s="3">
         <f t="shared" si="2"/>
         <v>17.413352542829998</v>
       </c>
-      <c r="Y29" s="5">
+      <c r="Y29" s="3">
         <f t="shared" si="3"/>
         <v>4.4931655974515483E-2</v>
       </c>
-      <c r="Z29" s="5">
+      <c r="Z29" s="3">
         <f t="shared" si="4"/>
         <v>0.26897862077594109</v>
       </c>
@@ -40156,55 +40150,55 @@
       <c r="H30">
         <v>532</v>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="3">
         <f t="shared" si="5"/>
         <v>11910.556731430001</v>
       </c>
-      <c r="J30" s="5">
+      <c r="J30" s="3">
         <f t="shared" si="6"/>
         <v>143.33333329999999</v>
       </c>
-      <c r="K30" s="9"/>
-      <c r="L30" s="5">
+      <c r="K30" s="7"/>
+      <c r="L30" s="3">
         <f t="shared" si="7"/>
         <v>83.096907447906261</v>
       </c>
-      <c r="M30" s="5">
+      <c r="M30" s="3">
         <v>94.276032310000005</v>
       </c>
-      <c r="N30" s="5"/>
-      <c r="O30" s="5">
+      <c r="N30" s="3"/>
+      <c r="O30" s="3">
         <v>102.3</v>
       </c>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5">
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3">
         <v>101.6</v>
       </c>
-      <c r="R30" s="5">
+      <c r="R30" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S30" s="5">
+      <c r="S30" s="3">
         <v>102.7</v>
       </c>
-      <c r="T30" s="5"/>
-      <c r="U30" s="9"/>
-      <c r="V30" s="5">
+      <c r="T30" s="3"/>
+      <c r="U30" s="7"/>
+      <c r="V30" s="3">
         <f t="shared" si="0"/>
         <v>67.16730527708512</v>
       </c>
-      <c r="W30" s="5">
+      <c r="W30" s="3">
         <f t="shared" si="1"/>
         <v>3.715275532270367</v>
       </c>
-      <c r="X30" s="5">
+      <c r="X30" s="3">
         <f t="shared" si="2"/>
         <v>17.250932986012582</v>
       </c>
-      <c r="Y30" s="5">
+      <c r="Y30" s="3">
         <f t="shared" si="3"/>
         <v>4.513642914620121E-2</v>
       </c>
-      <c r="Z30" s="5">
+      <c r="Z30" s="3">
         <f t="shared" si="4"/>
         <v>0.2517814415078104</v>
       </c>
@@ -40249,55 +40243,55 @@
       <c r="H31">
         <v>532</v>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="3">
         <f t="shared" si="5"/>
         <v>11857.71451071</v>
       </c>
-      <c r="J31" s="5">
+      <c r="J31" s="3">
         <f t="shared" si="6"/>
         <v>144.55555560000002</v>
       </c>
-      <c r="K31" s="9"/>
-      <c r="L31" s="5">
+      <c r="K31" s="7"/>
+      <c r="L31" s="3">
         <f t="shared" si="7"/>
         <v>82.02877060997578</v>
       </c>
-      <c r="M31" s="5">
+      <c r="M31" s="3">
         <v>92.273989950000001</v>
       </c>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5">
+      <c r="N31" s="3"/>
+      <c r="O31" s="3">
         <v>102.3</v>
       </c>
-      <c r="P31" s="5"/>
-      <c r="Q31" s="5">
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3">
         <v>101.6</v>
       </c>
-      <c r="R31" s="5">
+      <c r="R31" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S31" s="5">
+      <c r="S31" s="3">
         <v>102.7</v>
       </c>
-      <c r="T31" s="5"/>
-      <c r="U31" s="9"/>
-      <c r="V31" s="5">
+      <c r="T31" s="3"/>
+      <c r="U31" s="7"/>
+      <c r="V31" s="3">
         <f t="shared" si="0"/>
         <v>67.466626834153615</v>
       </c>
-      <c r="W31" s="5">
+      <c r="W31" s="3">
         <f t="shared" si="1"/>
         <v>3.5354199126767352</v>
       </c>
-      <c r="X31" s="5">
+      <c r="X31" s="3">
         <f t="shared" si="2"/>
         <v>17.097090869989334</v>
       </c>
-      <c r="Y31" s="5">
+      <c r="Y31" s="3">
         <f t="shared" si="3"/>
         <v>4.5337573232551227E-2</v>
       </c>
-      <c r="Z31" s="5">
+      <c r="Z31" s="3">
         <f t="shared" si="4"/>
         <v>0.23439833776480232</v>
       </c>
@@ -40342,55 +40336,55 @@
       <c r="H32">
         <v>532</v>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="3">
         <f t="shared" si="5"/>
         <v>11829.49639</v>
       </c>
-      <c r="J32" s="5">
+      <c r="J32" s="3">
         <f t="shared" si="6"/>
         <v>145.7777778</v>
       </c>
-      <c r="K32" s="9"/>
-      <c r="L32" s="5">
+      <c r="K32" s="7"/>
+      <c r="L32" s="3">
         <f t="shared" si="7"/>
         <v>81.147459980008009</v>
       </c>
-      <c r="M32" s="5">
+      <c r="M32" s="3">
         <v>90.314462890000001</v>
       </c>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5">
+      <c r="N32" s="3"/>
+      <c r="O32" s="3">
         <v>102.3</v>
       </c>
-      <c r="P32" s="5"/>
-      <c r="Q32" s="5">
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3">
         <v>101.6</v>
       </c>
-      <c r="R32" s="5">
+      <c r="R32" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S32" s="5">
+      <c r="S32" s="3">
         <v>102.7</v>
       </c>
-      <c r="T32" s="5"/>
-      <c r="U32" s="9"/>
-      <c r="V32" s="5">
+      <c r="T32" s="3"/>
+      <c r="U32" s="7"/>
+      <c r="V32" s="3">
         <f t="shared" si="0"/>
         <v>67.627561954055423</v>
       </c>
-      <c r="W32" s="5">
+      <c r="W32" s="3">
         <f t="shared" si="1"/>
         <v>3.5438533152973899</v>
       </c>
-      <c r="X32" s="5">
+      <c r="X32" s="3">
         <f t="shared" si="2"/>
         <v>16.917883264175035</v>
       </c>
-      <c r="Y32" s="5">
+      <c r="Y32" s="3">
         <f t="shared" si="3"/>
         <v>4.5445721633125248E-2</v>
       </c>
-      <c r="Z32" s="5">
+      <c r="Z32" s="3">
         <f t="shared" si="4"/>
         <v>0.21640819825297736</v>
       </c>
@@ -40438,57 +40432,57 @@
       <c r="H33">
         <v>532</v>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="3">
         <f t="shared" si="5"/>
         <v>11802.07407517</v>
       </c>
-      <c r="J33" s="5">
+      <c r="J33" s="3">
         <f t="shared" si="6"/>
         <v>147</v>
       </c>
-      <c r="K33" s="9"/>
-      <c r="L33" s="5">
+      <c r="K33" s="7"/>
+      <c r="L33" s="3">
         <f t="shared" si="7"/>
         <v>80.286218198435378</v>
       </c>
-      <c r="M33" s="5">
+      <c r="M33" s="3">
         <v>88.396548280000005</v>
       </c>
-      <c r="N33" s="5">
+      <c r="N33" s="3">
         <v>95</v>
       </c>
-      <c r="O33" s="5">
+      <c r="O33" s="3">
         <v>102.3</v>
       </c>
-      <c r="P33" s="5"/>
-      <c r="Q33" s="5">
+      <c r="P33" s="3"/>
+      <c r="Q33" s="3">
         <v>101.6</v>
       </c>
-      <c r="R33" s="5">
+      <c r="R33" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S33" s="5">
+      <c r="S33" s="3">
         <v>102.7</v>
       </c>
-      <c r="T33" s="5"/>
-      <c r="U33" s="9"/>
-      <c r="V33" s="5">
+      <c r="T33" s="3"/>
+      <c r="U33" s="7"/>
+      <c r="V33" s="3">
         <f t="shared" si="0"/>
         <v>67.784695715738138</v>
       </c>
-      <c r="W33" s="5">
+      <c r="W33" s="3">
         <f t="shared" si="1"/>
         <v>3.5520875172439679</v>
       </c>
-      <c r="X33" s="5">
+      <c r="X33" s="3">
         <f t="shared" si="2"/>
         <v>16.837300345205438</v>
       </c>
-      <c r="Y33" s="5">
+      <c r="Y33" s="3">
         <f t="shared" si="3"/>
         <v>4.5551315520976028E-2</v>
       </c>
-      <c r="Z33" s="5">
+      <c r="Z33" s="3">
         <f t="shared" si="4"/>
         <v>0.10445126925559001</v>
       </c>
@@ -40539,55 +40533,55 @@
       <c r="H34">
         <v>532</v>
       </c>
-      <c r="I34" s="5">
+      <c r="I34" s="3">
         <f t="shared" si="5"/>
         <v>11779.461976809998</v>
       </c>
-      <c r="J34" s="5">
+      <c r="J34" s="3">
         <f t="shared" si="6"/>
         <v>151</v>
       </c>
-      <c r="K34" s="9"/>
-      <c r="L34" s="5">
+      <c r="K34" s="7"/>
+      <c r="L34" s="3">
         <f t="shared" si="7"/>
         <v>78.009681965629127</v>
       </c>
-      <c r="M34" s="5">
+      <c r="M34" s="3">
         <v>86.519362419999993</v>
       </c>
-      <c r="N34" s="5"/>
-      <c r="O34" s="5">
+      <c r="N34" s="3"/>
+      <c r="O34" s="3">
         <v>102.3</v>
       </c>
-      <c r="P34" s="5"/>
-      <c r="Q34" s="5">
+      <c r="P34" s="3"/>
+      <c r="Q34" s="3">
         <v>101.6</v>
       </c>
-      <c r="R34" s="5">
+      <c r="R34" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S34" s="5">
+      <c r="S34" s="3">
         <v>102.7</v>
       </c>
-      <c r="T34" s="5"/>
-      <c r="U34" s="9"/>
-      <c r="V34" s="5">
+      <c r="T34" s="3"/>
+      <c r="U34" s="7"/>
+      <c r="V34" s="3">
         <f t="shared" si="0"/>
         <v>67.914816616832312</v>
       </c>
-      <c r="W34" s="5">
+      <c r="W34" s="3">
         <f t="shared" si="1"/>
         <v>3.5589061777635553</v>
       </c>
-      <c r="X34" s="5">
+      <c r="X34" s="3">
         <f t="shared" si="2"/>
         <v>16.695101472984032</v>
       </c>
-      <c r="Y34" s="5">
+      <c r="Y34" s="3">
         <f t="shared" si="3"/>
         <v>4.5638756766511315E-2</v>
       </c>
-      <c r="Z34" s="5">
+      <c r="Z34" s="3">
         <f t="shared" si="4"/>
         <v>8.7209813404245107E-2</v>
       </c>
@@ -40635,59 +40629,59 @@
       <c r="H35">
         <v>532</v>
       </c>
-      <c r="I35" s="5">
+      <c r="I35" s="3">
         <f t="shared" si="5"/>
         <v>11853.800475448999</v>
       </c>
-      <c r="J35" s="5">
+      <c r="J35" s="3">
         <f t="shared" si="6"/>
         <v>154</v>
       </c>
-      <c r="K35" s="9"/>
-      <c r="L35" s="5">
+      <c r="K35" s="7"/>
+      <c r="L35" s="3">
         <f t="shared" si="7"/>
         <v>76.972730360058435</v>
       </c>
-      <c r="M35" s="5">
+      <c r="M35" s="3">
         <v>84.682040420000007</v>
       </c>
-      <c r="N35" s="5">
+      <c r="N35" s="3">
         <v>78</v>
       </c>
-      <c r="O35" s="5">
+      <c r="O35" s="3">
         <v>102.3</v>
       </c>
-      <c r="P35" s="5">
+      <c r="P35" s="3">
         <v>102</v>
       </c>
-      <c r="Q35" s="5">
+      <c r="Q35" s="3">
         <v>101.6</v>
       </c>
-      <c r="R35" s="5">
+      <c r="R35" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S35" s="5">
+      <c r="S35" s="3">
         <v>102.7</v>
       </c>
-      <c r="T35" s="5"/>
-      <c r="U35" s="9"/>
-      <c r="V35" s="5">
+      <c r="T35" s="3"/>
+      <c r="U35" s="7"/>
+      <c r="V35" s="3">
         <f t="shared" si="0"/>
         <v>68.163792842092235</v>
       </c>
-      <c r="W35" s="5">
+      <c r="W35" s="3">
         <f t="shared" si="1"/>
         <v>3.53658728159182</v>
       </c>
-      <c r="X35" s="5">
+      <c r="X35" s="3">
         <f t="shared" si="2"/>
         <v>16.559973335687904</v>
       </c>
-      <c r="Y35" s="5">
+      <c r="Y35" s="3">
         <f t="shared" si="3"/>
         <v>4.5352543356322758E-2</v>
       </c>
-      <c r="Z35" s="5">
+      <c r="Z35" s="3">
         <f t="shared" si="4"/>
         <v>6.9330317023821073E-2</v>
       </c>
@@ -40735,57 +40729,57 @@
       <c r="H36">
         <v>532</v>
       </c>
-      <c r="I36" s="5">
+      <c r="I36" s="3">
         <f t="shared" si="5"/>
         <v>11587.806922214</v>
       </c>
-      <c r="J36" s="5">
+      <c r="J36" s="3">
         <f t="shared" si="6"/>
         <v>160</v>
       </c>
-      <c r="K36" s="9"/>
-      <c r="L36" s="5">
+      <c r="K36" s="7"/>
+      <c r="L36" s="3">
         <f t="shared" si="7"/>
         <v>72.423793263837496</v>
       </c>
-      <c r="M36" s="5">
+      <c r="M36" s="3">
         <v>82.883735720000004</v>
       </c>
-      <c r="N36" s="5"/>
-      <c r="O36" s="5">
+      <c r="N36" s="3"/>
+      <c r="O36" s="3">
         <v>102.3</v>
       </c>
-      <c r="P36" s="5">
+      <c r="P36" s="3">
         <v>102</v>
       </c>
-      <c r="Q36" s="5">
+      <c r="Q36" s="3">
         <v>101.6</v>
       </c>
-      <c r="R36" s="5">
+      <c r="R36" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S36" s="5">
+      <c r="S36" s="3">
         <v>102.7</v>
       </c>
-      <c r="T36" s="5"/>
-      <c r="U36" s="9"/>
-      <c r="V36" s="5">
+      <c r="T36" s="3"/>
+      <c r="U36" s="7"/>
+      <c r="V36" s="3">
         <f t="shared" si="0"/>
         <v>70.418846765190381</v>
       </c>
-      <c r="W36" s="5">
+      <c r="W36" s="3">
         <f t="shared" si="1"/>
         <v>3.6177682525616559</v>
       </c>
-      <c r="X36" s="5">
+      <c r="X36" s="3">
         <f t="shared" si="2"/>
         <v>13.975535999788487</v>
       </c>
-      <c r="Y36" s="5">
+      <c r="Y36" s="3">
         <f t="shared" si="3"/>
         <v>4.6393593162948957E-2</v>
       </c>
-      <c r="Z36" s="5">
+      <c r="Z36" s="3">
         <f t="shared" si="4"/>
         <v>4.9645237037664186E-2</v>
       </c>
@@ -40833,57 +40827,57 @@
       <c r="H37">
         <v>532</v>
       </c>
-      <c r="I37" s="5">
+      <c r="I37" s="3">
         <f t="shared" si="5"/>
         <v>11695.467606342001</v>
       </c>
-      <c r="J37" s="5">
+      <c r="J37" s="3">
         <f t="shared" si="6"/>
         <v>163</v>
       </c>
-      <c r="K37" s="9"/>
-      <c r="L37" s="5">
+      <c r="K37" s="7"/>
+      <c r="L37" s="3">
         <f t="shared" si="7"/>
         <v>71.751335008233141</v>
       </c>
-      <c r="M37" s="5">
+      <c r="M37" s="3">
         <v>81.123619750000003</v>
       </c>
-      <c r="N37" s="5"/>
-      <c r="O37" s="5">
+      <c r="N37" s="3"/>
+      <c r="O37" s="3">
         <v>102.3</v>
       </c>
-      <c r="P37" s="5">
+      <c r="P37" s="3">
         <v>102</v>
       </c>
-      <c r="Q37" s="5">
+      <c r="Q37" s="3">
         <v>101.6</v>
       </c>
-      <c r="R37" s="5">
+      <c r="R37" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S37" s="5">
+      <c r="S37" s="3">
         <v>102.7</v>
       </c>
-      <c r="T37" s="5"/>
-      <c r="U37" s="9"/>
-      <c r="V37" s="5">
+      <c r="T37" s="3"/>
+      <c r="U37" s="7"/>
+      <c r="V37" s="3">
         <f t="shared" si="0"/>
         <v>70.905245340538485</v>
       </c>
-      <c r="W37" s="5">
+      <c r="W37" s="3">
         <f t="shared" si="1"/>
         <v>3.5844654879183557</v>
       </c>
-      <c r="X37" s="5">
+      <c r="X37" s="3">
         <f t="shared" si="2"/>
         <v>13.618435616343538</v>
       </c>
-      <c r="Y37" s="5">
+      <c r="Y37" s="3">
         <f t="shared" si="3"/>
         <v>4.5966524648273173E-2</v>
       </c>
-      <c r="Z37" s="5">
+      <c r="Z37" s="3">
         <f t="shared" si="4"/>
         <v>4.5674790626612519E-2</v>
       </c>
@@ -40931,59 +40925,59 @@
       <c r="H38">
         <v>532</v>
       </c>
-      <c r="I38" s="5">
+      <c r="I38" s="3">
         <f t="shared" si="5"/>
         <v>11532.713136597</v>
       </c>
-      <c r="J38" s="5">
+      <c r="J38" s="3">
         <f t="shared" si="6"/>
         <v>170</v>
       </c>
-      <c r="K38" s="9"/>
-      <c r="L38" s="5">
+      <c r="K38" s="7"/>
+      <c r="L38" s="3">
         <f t="shared" si="7"/>
         <v>67.83948903880588</v>
       </c>
-      <c r="M38" s="5">
+      <c r="M38" s="3">
         <v>79.40088154</v>
       </c>
-      <c r="N38" s="5">
+      <c r="N38" s="3">
         <v>65</v>
       </c>
-      <c r="O38" s="5">
+      <c r="O38" s="3">
         <v>102.3</v>
       </c>
-      <c r="P38" s="5">
+      <c r="P38" s="3">
         <v>102</v>
       </c>
-      <c r="Q38" s="5">
+      <c r="Q38" s="3">
         <v>101.6</v>
       </c>
-      <c r="R38" s="5">
+      <c r="R38" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S38" s="5">
+      <c r="S38" s="3">
         <v>102.7</v>
       </c>
-      <c r="T38" s="5"/>
-      <c r="U38" s="9"/>
-      <c r="V38" s="5">
+      <c r="T38" s="3"/>
+      <c r="U38" s="7"/>
+      <c r="V38" s="3">
         <f t="shared" si="0"/>
         <v>71.324608551107843</v>
       </c>
-      <c r="W38" s="5">
+      <c r="W38" s="3">
         <f t="shared" si="1"/>
         <v>3.6350509635905226</v>
       </c>
-      <c r="X38" s="5">
+      <c r="X38" s="3">
         <f t="shared" si="2"/>
         <v>12.965226883647318</v>
       </c>
-      <c r="Y38" s="5">
+      <c r="Y38" s="3">
         <f t="shared" si="3"/>
         <v>5.0189057262096555E-2</v>
       </c>
-      <c r="Z38" s="5">
+      <c r="Z38" s="3">
         <f t="shared" si="4"/>
         <v>3.919331508087566E-2</v>
       </c>
@@ -41034,57 +41028,57 @@
       <c r="H39">
         <v>532</v>
       </c>
-      <c r="I39" s="5">
+      <c r="I39" s="3">
         <f t="shared" si="5"/>
         <v>11385.743893008999</v>
       </c>
-      <c r="J39" s="5">
+      <c r="J39" s="3">
         <f t="shared" si="6"/>
         <v>175</v>
       </c>
-      <c r="K39" s="9"/>
-      <c r="L39" s="5">
+      <c r="K39" s="7"/>
+      <c r="L39" s="3">
         <f t="shared" si="7"/>
         <v>65.06139367433714</v>
       </c>
-      <c r="M39" s="5">
+      <c r="M39" s="3">
         <v>77.714727339999996</v>
       </c>
-      <c r="N39" s="5"/>
-      <c r="O39" s="5">
+      <c r="N39" s="3"/>
+      <c r="O39" s="3">
         <v>102.3</v>
       </c>
-      <c r="P39" s="5">
+      <c r="P39" s="3">
         <v>102</v>
       </c>
-      <c r="Q39" s="5">
+      <c r="Q39" s="3">
         <v>101.6</v>
       </c>
-      <c r="R39" s="5">
+      <c r="R39" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S39" s="5">
+      <c r="S39" s="3">
         <v>102.7</v>
       </c>
-      <c r="T39" s="5"/>
-      <c r="U39" s="9"/>
-      <c r="V39" s="5">
+      <c r="T39" s="3"/>
+      <c r="U39" s="7"/>
+      <c r="V39" s="3">
         <f t="shared" si="0"/>
         <v>71.658800484785772</v>
       </c>
-      <c r="W39" s="5">
+      <c r="W39" s="3">
         <f t="shared" si="1"/>
         <v>3.6819728595635004</v>
       </c>
-      <c r="X39" s="5">
+      <c r="X39" s="3">
         <f t="shared" si="2"/>
         <v>12.406095985237382</v>
       </c>
-      <c r="Y39" s="5">
+      <c r="Y39" s="3">
         <f t="shared" si="3"/>
         <v>5.4456872192664374E-2</v>
       </c>
-      <c r="Z39" s="5">
+      <c r="Z39" s="3">
         <f t="shared" si="4"/>
         <v>3.6007809832410746E-2</v>
       </c>
@@ -41132,57 +41126,57 @@
       <c r="H40">
         <v>532</v>
       </c>
-      <c r="I40" s="5">
+      <c r="I40" s="3">
         <f t="shared" si="5"/>
         <v>11480.063846300998</v>
       </c>
-      <c r="J40" s="5">
+      <c r="J40" s="3">
         <f t="shared" si="6"/>
         <v>177</v>
       </c>
-      <c r="K40" s="9"/>
-      <c r="L40" s="5">
+      <c r="K40" s="7"/>
+      <c r="L40" s="3">
         <f t="shared" si="7"/>
         <v>64.859117775711852</v>
       </c>
-      <c r="M40" s="5">
+      <c r="M40" s="3">
         <v>76.064380240000006</v>
       </c>
-      <c r="N40" s="5"/>
-      <c r="O40" s="5">
+      <c r="N40" s="3"/>
+      <c r="O40" s="3">
         <v>102.3</v>
       </c>
-      <c r="P40" s="5">
+      <c r="P40" s="3">
         <v>102</v>
       </c>
-      <c r="Q40" s="5">
+      <c r="Q40" s="3">
         <v>101.6</v>
       </c>
-      <c r="R40" s="5">
+      <c r="R40" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S40" s="5">
+      <c r="S40" s="3">
         <v>102.7</v>
       </c>
-      <c r="T40" s="5"/>
-      <c r="U40" s="9"/>
-      <c r="V40" s="5">
+      <c r="T40" s="3"/>
+      <c r="U40" s="7"/>
+      <c r="V40" s="3">
         <f t="shared" si="0"/>
         <v>72.209964256174828</v>
       </c>
-      <c r="W40" s="5">
+      <c r="W40" s="3">
         <f t="shared" si="1"/>
         <v>3.6517218511382872</v>
       </c>
-      <c r="X40" s="5">
+      <c r="X40" s="3">
         <f t="shared" si="2"/>
         <v>12.019278938458111</v>
       </c>
-      <c r="Y40" s="5">
+      <c r="Y40" s="3">
         <f t="shared" si="3"/>
         <v>6.2750870521692745E-2</v>
       </c>
-      <c r="Z40" s="5">
+      <c r="Z40" s="3">
         <f t="shared" si="4"/>
         <v>3.5532122082355268E-2</v>
       </c>
@@ -41230,57 +41224,57 @@
       <c r="H41">
         <v>532</v>
       </c>
-      <c r="I41" s="5">
+      <c r="I41" s="3">
         <f t="shared" si="5"/>
         <v>11515.394229122998</v>
       </c>
-      <c r="J41" s="5">
+      <c r="J41" s="3">
         <f t="shared" si="6"/>
         <v>184</v>
       </c>
-      <c r="K41" s="9"/>
-      <c r="L41" s="5">
+      <c r="K41" s="7"/>
+      <c r="L41" s="3">
         <f t="shared" si="7"/>
         <v>62.583664288711944</v>
       </c>
-      <c r="M41" s="5">
+      <c r="M41" s="3">
         <v>74.449079859999998</v>
       </c>
-      <c r="N41" s="5"/>
-      <c r="O41" s="5">
+      <c r="N41" s="3"/>
+      <c r="O41" s="3">
         <v>102.3</v>
       </c>
-      <c r="P41" s="5">
+      <c r="P41" s="3">
         <v>102</v>
       </c>
-      <c r="Q41" s="5">
+      <c r="Q41" s="3">
         <v>101.6</v>
       </c>
-      <c r="R41" s="5">
+      <c r="R41" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S41" s="5">
+      <c r="S41" s="3">
         <v>102.7</v>
       </c>
-      <c r="T41" s="5"/>
-      <c r="U41" s="9"/>
-      <c r="V41" s="5">
+      <c r="T41" s="3"/>
+      <c r="U41" s="7"/>
+      <c r="V41" s="3">
         <f t="shared" si="0"/>
         <v>72.512932113796495</v>
       </c>
-      <c r="W41" s="5">
+      <c r="W41" s="3">
         <f t="shared" si="1"/>
         <v>3.5678761849153848</v>
       </c>
-      <c r="X41" s="5">
+      <c r="X41" s="3">
         <f t="shared" si="2"/>
         <v>11.824750763254618</v>
       </c>
-      <c r="Y41" s="5">
+      <c r="Y41" s="3">
         <f t="shared" si="3"/>
         <v>6.4736993381838775E-2</v>
       </c>
-      <c r="Z41" s="5">
+      <c r="Z41" s="3">
         <f t="shared" si="4"/>
         <v>3.7452767462295221E-2</v>
       </c>
@@ -41328,57 +41322,57 @@
       <c r="H42">
         <v>532</v>
       </c>
-      <c r="I42" s="5">
+      <c r="I42" s="3">
         <f t="shared" si="5"/>
         <v>11749.006155509998</v>
       </c>
-      <c r="J42" s="5">
+      <c r="J42" s="3">
         <f t="shared" si="6"/>
         <v>192</v>
       </c>
-      <c r="K42" s="9"/>
-      <c r="L42" s="5">
+      <c r="K42" s="7"/>
+      <c r="L42" s="3">
         <f t="shared" si="7"/>
         <v>61.192740393281241</v>
       </c>
-      <c r="M42" s="5">
+      <c r="M42" s="3">
         <v>72.868081930000002</v>
       </c>
-      <c r="N42" s="5"/>
-      <c r="O42" s="5">
+      <c r="N42" s="3"/>
+      <c r="O42" s="3">
         <v>102.3</v>
       </c>
-      <c r="P42" s="5">
+      <c r="P42" s="3">
         <v>102</v>
       </c>
-      <c r="Q42" s="5">
+      <c r="Q42" s="3">
         <v>101.6</v>
       </c>
-      <c r="R42" s="5">
+      <c r="R42" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S42" s="5">
+      <c r="S42" s="3">
         <v>102.7</v>
       </c>
-      <c r="T42" s="5"/>
-      <c r="U42" s="9"/>
-      <c r="V42" s="5">
+      <c r="T42" s="3"/>
+      <c r="U42" s="7"/>
+      <c r="V42" s="3">
         <f t="shared" si="0"/>
         <v>73.26151579181267</v>
       </c>
-      <c r="W42" s="5">
+      <c r="W42" s="3">
         <f t="shared" si="1"/>
         <v>3.4227632650563029</v>
       </c>
-      <c r="X42" s="5">
+      <c r="X42" s="3">
         <f t="shared" si="2"/>
         <v>11.436261426843004</v>
       </c>
-      <c r="Y42" s="5">
+      <c r="Y42" s="3">
         <f t="shared" si="3"/>
         <v>7.0313351535063545E-2</v>
       </c>
-      <c r="Z42" s="5">
+      <c r="Z42" s="3">
         <f t="shared" si="4"/>
         <v>3.5299239400389731E-2</v>
       </c>
@@ -41426,61 +41420,61 @@
       <c r="H43">
         <v>532</v>
       </c>
-      <c r="I43" s="5">
+      <c r="I43" s="3">
         <f t="shared" si="5"/>
         <v>12092.466287744999</v>
       </c>
-      <c r="J43" s="5">
+      <c r="J43" s="3">
         <f t="shared" si="6"/>
         <v>202.52588490000002</v>
       </c>
-      <c r="K43" s="9"/>
-      <c r="L43" s="5">
+      <c r="K43" s="7"/>
+      <c r="L43" s="3">
         <f t="shared" si="7"/>
         <v>59.708250595798276</v>
       </c>
-      <c r="M43" s="5">
+      <c r="M43" s="3">
         <v>71.320658019999996</v>
       </c>
-      <c r="N43" s="5">
+      <c r="N43" s="3">
         <v>65</v>
       </c>
-      <c r="O43" s="5">
+      <c r="O43" s="3">
         <v>102.3</v>
       </c>
-      <c r="P43" s="5">
+      <c r="P43" s="3">
         <v>102</v>
       </c>
-      <c r="Q43" s="5">
+      <c r="Q43" s="3">
         <v>101.6</v>
       </c>
-      <c r="R43" s="5">
+      <c r="R43" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S43" s="5">
+      <c r="S43" s="3">
         <v>102.7</v>
       </c>
-      <c r="T43" s="5">
+      <c r="T43" s="3">
         <v>76</v>
       </c>
-      <c r="U43" s="9"/>
-      <c r="V43" s="5">
+      <c r="U43" s="7"/>
+      <c r="V43" s="3">
         <f t="shared" si="0"/>
         <v>74.223899297500125</v>
       </c>
-      <c r="W43" s="5">
+      <c r="W43" s="3">
         <f t="shared" si="1"/>
         <v>3.1428988450864019</v>
       </c>
-      <c r="X43" s="5">
+      <c r="X43" s="3">
         <f t="shared" si="2"/>
         <v>11.111439362553419</v>
       </c>
-      <c r="Y43" s="5">
+      <c r="Y43" s="3">
         <f t="shared" si="3"/>
         <v>6.8019871251043598E-2</v>
       </c>
-      <c r="Z43" s="5">
+      <c r="Z43" s="3">
         <f t="shared" si="4"/>
         <v>2.9728968098453872E-2</v>
       </c>
@@ -41531,59 +41525,59 @@
       <c r="H44">
         <v>520</v>
       </c>
-      <c r="I44" s="5">
+      <c r="I44" s="3">
         <f t="shared" si="5"/>
         <v>12047.313171469001</v>
       </c>
-      <c r="J44" s="5">
+      <c r="J44" s="3">
         <f t="shared" si="6"/>
         <v>208.94864799999999</v>
       </c>
-      <c r="K44" s="9"/>
-      <c r="L44" s="5">
+      <c r="K44" s="7"/>
+      <c r="L44" s="3">
         <f t="shared" si="7"/>
         <v>57.656813225558658</v>
       </c>
-      <c r="M44" s="5">
+      <c r="M44" s="3">
         <v>69.806095139999996</v>
       </c>
-      <c r="N44" s="5"/>
-      <c r="O44" s="5">
+      <c r="N44" s="3"/>
+      <c r="O44" s="3">
         <v>102.3</v>
       </c>
-      <c r="P44" s="5">
+      <c r="P44" s="3">
         <v>102</v>
       </c>
-      <c r="Q44" s="5">
+      <c r="Q44" s="3">
         <v>101.6</v>
       </c>
-      <c r="R44" s="5">
+      <c r="R44" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S44" s="5">
+      <c r="S44" s="3">
         <v>102.7</v>
       </c>
-      <c r="T44" s="5">
+      <c r="T44" s="3">
         <v>76</v>
       </c>
-      <c r="U44" s="9"/>
-      <c r="V44" s="5">
+      <c r="U44" s="7"/>
+      <c r="V44" s="3">
         <f t="shared" si="0"/>
         <v>74.9295703657655</v>
       </c>
-      <c r="W44" s="5">
+      <c r="W44" s="3">
         <f t="shared" si="1"/>
         <v>3.0494794679202579</v>
       </c>
-      <c r="X44" s="5">
+      <c r="X44" s="3">
         <f t="shared" si="2"/>
         <v>10.559835648772097</v>
       </c>
-      <c r="Y44" s="5">
+      <c r="Y44" s="3">
         <f t="shared" si="3"/>
         <v>6.8646675671929766E-2</v>
       </c>
-      <c r="Z44" s="5">
+      <c r="Z44" s="3">
         <f t="shared" si="4"/>
         <v>2.7734639429088385E-2</v>
       </c>
@@ -41631,59 +41625,59 @@
       <c r="H45">
         <v>510</v>
       </c>
-      <c r="I45" s="5">
+      <c r="I45" s="3">
         <f t="shared" si="5"/>
         <v>12072.594883022</v>
       </c>
-      <c r="J45" s="5">
+      <c r="J45" s="3">
         <f t="shared" si="6"/>
         <v>213.6288232</v>
       </c>
-      <c r="K45" s="9"/>
-      <c r="L45" s="5">
+      <c r="K45" s="7"/>
+      <c r="L45" s="3">
         <f t="shared" si="7"/>
         <v>56.512013230160413</v>
       </c>
-      <c r="M45" s="5">
+      <c r="M45" s="3">
         <v>68.323695470000004</v>
       </c>
-      <c r="N45" s="5"/>
-      <c r="O45" s="5">
+      <c r="N45" s="3"/>
+      <c r="O45" s="3">
         <v>102.3</v>
       </c>
-      <c r="P45" s="5">
+      <c r="P45" s="3">
         <v>102</v>
       </c>
-      <c r="Q45" s="5">
+      <c r="Q45" s="3">
         <v>101.6</v>
       </c>
-      <c r="R45" s="5">
+      <c r="R45" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S45" s="5">
+      <c r="S45" s="3">
         <v>102.7</v>
       </c>
-      <c r="T45" s="5">
+      <c r="T45" s="3">
         <v>76</v>
       </c>
-      <c r="U45" s="9"/>
-      <c r="V45" s="5">
+      <c r="U45" s="7"/>
+      <c r="V45" s="3">
         <f t="shared" si="0"/>
         <v>75.431173564903631</v>
       </c>
-      <c r="W45" s="5">
+      <c r="W45" s="3">
         <f t="shared" si="1"/>
         <v>2.9381148248321756</v>
       </c>
-      <c r="X45" s="5">
+      <c r="X45" s="3">
         <f t="shared" si="2"/>
         <v>10.360119809527786</v>
       </c>
-      <c r="Y45" s="5">
+      <c r="Y45" s="3">
         <f t="shared" si="3"/>
         <v>6.8874008285438534E-2</v>
       </c>
-      <c r="Z45" s="5">
+      <c r="Z45" s="3">
         <f t="shared" si="4"/>
         <v>2.5625261610912303E-2</v>
       </c>
@@ -41731,59 +41725,59 @@
       <c r="H46">
         <v>500</v>
       </c>
-      <c r="I46" s="5">
+      <c r="I46" s="3">
         <f t="shared" si="5"/>
         <v>12101.860575282</v>
       </c>
-      <c r="J46" s="5">
+      <c r="J46" s="3">
         <f t="shared" si="6"/>
         <v>217.3311205</v>
       </c>
-      <c r="K46" s="9"/>
-      <c r="L46" s="5">
+      <c r="K46" s="7"/>
+      <c r="L46" s="3">
         <f t="shared" si="7"/>
         <v>55.683974515200646</v>
       </c>
-      <c r="M46" s="5">
+      <c r="M46" s="3">
         <v>66.87277598</v>
       </c>
-      <c r="N46" s="5"/>
-      <c r="O46" s="5">
+      <c r="N46" s="3"/>
+      <c r="O46" s="3">
         <v>102.3</v>
       </c>
-      <c r="P46" s="5">
+      <c r="P46" s="3">
         <v>102</v>
       </c>
-      <c r="Q46" s="5">
+      <c r="Q46" s="3">
         <v>101.6</v>
       </c>
-      <c r="R46" s="5">
+      <c r="R46" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S46" s="5">
+      <c r="S46" s="3">
         <v>102.7</v>
       </c>
-      <c r="T46" s="5">
+      <c r="T46" s="3">
         <v>76</v>
       </c>
-      <c r="U46" s="9"/>
-      <c r="V46" s="5">
+      <c r="U46" s="7"/>
+      <c r="V46" s="3">
         <f t="shared" si="0"/>
         <v>75.885438795728334</v>
       </c>
-      <c r="W46" s="5">
+      <c r="W46" s="3">
         <f t="shared" si="1"/>
         <v>2.879689707480201</v>
       </c>
-      <c r="X46" s="5">
+      <c r="X46" s="3">
         <f t="shared" si="2"/>
         <v>10.157893576387982</v>
       </c>
-      <c r="Y46" s="5">
+      <c r="Y46" s="3">
         <f t="shared" si="3"/>
         <v>6.929975723839947E-2</v>
       </c>
-      <c r="Z46" s="5">
+      <c r="Z46" s="3">
         <f t="shared" si="4"/>
         <v>2.395386943988528E-2</v>
       </c>
@@ -41831,59 +41825,59 @@
       <c r="H47">
         <v>490</v>
       </c>
-      <c r="I47" s="5">
+      <c r="I47" s="3">
         <f t="shared" si="5"/>
         <v>11968.629252107001</v>
       </c>
-      <c r="J47" s="5">
+      <c r="J47" s="3">
         <f t="shared" si="6"/>
         <v>220.40369699999999</v>
       </c>
-      <c r="K47" s="9"/>
-      <c r="L47" s="5">
+      <c r="K47" s="7"/>
+      <c r="L47" s="3">
         <f t="shared" si="7"/>
         <v>54.303214578596659</v>
       </c>
-      <c r="M47" s="5">
+      <c r="M47" s="3">
         <v>65.452668169999995</v>
       </c>
-      <c r="N47" s="5"/>
-      <c r="O47" s="5">
+      <c r="N47" s="3"/>
+      <c r="O47" s="3">
         <v>102.3</v>
       </c>
-      <c r="P47" s="5">
+      <c r="P47" s="3">
         <v>102</v>
       </c>
-      <c r="Q47" s="5">
+      <c r="Q47" s="3">
         <v>101.6</v>
       </c>
-      <c r="R47" s="5">
+      <c r="R47" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S47" s="5">
+      <c r="S47" s="3">
         <v>102.7</v>
       </c>
-      <c r="T47" s="5">
+      <c r="T47" s="3">
         <v>76</v>
       </c>
-      <c r="U47" s="9"/>
-      <c r="V47" s="5">
+      <c r="U47" s="7"/>
+      <c r="V47" s="3">
         <f t="shared" si="0"/>
         <v>76.105833075215784</v>
       </c>
-      <c r="W47" s="5">
+      <c r="W47" s="3">
         <f t="shared" si="1"/>
         <v>2.8598543700377621</v>
       </c>
-      <c r="X47" s="5">
+      <c r="X47" s="3">
         <f t="shared" si="2"/>
         <v>10.151538446109917</v>
       </c>
-      <c r="Y47" s="5">
+      <c r="Y47" s="3">
         <f t="shared" si="3"/>
         <v>7.0670081108168512E-2</v>
       </c>
-      <c r="Z47" s="5">
+      <c r="Z47" s="3">
         <f t="shared" si="4"/>
         <v>2.2499614202068571E-2</v>
       </c>
@@ -41931,61 +41925,61 @@
       <c r="H48">
         <v>480</v>
       </c>
-      <c r="I48" s="5">
+      <c r="I48" s="3">
         <f t="shared" si="5"/>
         <v>11835.472545881999</v>
       </c>
-      <c r="J48" s="5">
+      <c r="J48" s="3">
         <f t="shared" si="6"/>
         <v>223.03538889999999</v>
       </c>
-      <c r="K48" s="9"/>
-      <c r="L48" s="5">
+      <c r="K48" s="7"/>
+      <c r="L48" s="3">
         <f t="shared" si="7"/>
         <v>53.065446717913204</v>
       </c>
-      <c r="M48" s="5">
+      <c r="M48" s="3">
         <v>64.062717710000001</v>
       </c>
-      <c r="N48" s="5">
+      <c r="N48" s="3">
         <v>65</v>
       </c>
-      <c r="O48" s="5">
+      <c r="O48" s="3">
         <v>102.3</v>
       </c>
-      <c r="P48" s="5">
+      <c r="P48" s="3">
         <v>102</v>
       </c>
-      <c r="Q48" s="5">
+      <c r="Q48" s="3">
         <v>101.6</v>
       </c>
-      <c r="R48" s="5">
+      <c r="R48" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S48" s="5">
+      <c r="S48" s="3">
         <v>102.7</v>
       </c>
-      <c r="T48" s="5">
+      <c r="T48" s="3">
         <v>76</v>
       </c>
-      <c r="U48" s="9"/>
-      <c r="V48" s="5">
+      <c r="U48" s="7"/>
+      <c r="V48" s="3">
         <f t="shared" si="0"/>
         <v>76.330708089414642</v>
       </c>
-      <c r="W48" s="5">
+      <c r="W48" s="3">
         <f t="shared" si="1"/>
         <v>2.8390188748053902</v>
       </c>
-      <c r="X48" s="5">
+      <c r="X48" s="3">
         <f t="shared" si="2"/>
         <v>10.144976276572667</v>
       </c>
-      <c r="Y48" s="5">
+      <c r="Y48" s="3">
         <f t="shared" si="3"/>
         <v>6.9244496163792704E-2</v>
       </c>
-      <c r="Z48" s="5">
+      <c r="Z48" s="3">
         <f t="shared" si="4"/>
         <v>2.1485842995637612E-2</v>
       </c>
@@ -42036,59 +42030,59 @@
       <c r="H49">
         <v>470</v>
       </c>
-      <c r="I49" s="5">
+      <c r="I49" s="3">
         <f t="shared" si="5"/>
         <v>11959.069885074001</v>
       </c>
-      <c r="J49" s="5">
+      <c r="J49" s="3">
         <f t="shared" si="6"/>
         <v>225.34045020000002</v>
       </c>
-      <c r="K49" s="9"/>
-      <c r="L49" s="5">
+      <c r="K49" s="7"/>
+      <c r="L49" s="3">
         <f t="shared" si="7"/>
         <v>53.071119164179251</v>
       </c>
-      <c r="M49" s="5">
+      <c r="M49" s="3">
         <v>62.70228419</v>
       </c>
-      <c r="N49" s="5"/>
-      <c r="O49" s="5">
+      <c r="N49" s="3"/>
+      <c r="O49" s="3">
         <v>102.3</v>
       </c>
-      <c r="P49" s="5">
+      <c r="P49" s="3">
         <v>102</v>
       </c>
-      <c r="Q49" s="5">
+      <c r="Q49" s="3">
         <v>101.6</v>
       </c>
-      <c r="R49" s="5">
+      <c r="R49" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S49" s="5">
+      <c r="S49" s="3">
         <v>102.7</v>
       </c>
-      <c r="T49" s="5">
+      <c r="T49" s="3">
         <v>76</v>
       </c>
-      <c r="U49" s="9"/>
-      <c r="V49" s="5">
+      <c r="U49" s="7"/>
+      <c r="V49" s="3">
         <f t="shared" si="0"/>
         <v>76.9726109259461</v>
       </c>
-      <c r="W49" s="5">
+      <c r="W49" s="3">
         <f t="shared" si="1"/>
         <v>2.7572146945268865</v>
       </c>
-      <c r="X49" s="5">
+      <c r="X49" s="3">
         <f t="shared" si="2"/>
         <v>9.9604441018167797</v>
       </c>
-      <c r="Y49" s="5">
+      <c r="Y49" s="3">
         <f t="shared" si="3"/>
         <v>6.6331133969712686E-2</v>
       </c>
-      <c r="Z49" s="5">
+      <c r="Z49" s="3">
         <f t="shared" si="4"/>
         <v>2.0079004722574553E-2</v>
       </c>
@@ -42136,59 +42130,59 @@
       <c r="H50">
         <v>460</v>
       </c>
-      <c r="I50" s="5">
+      <c r="I50" s="3">
         <f t="shared" si="5"/>
         <v>12080.381868788998</v>
       </c>
-      <c r="J50" s="5">
+      <c r="J50" s="3">
         <f t="shared" si="6"/>
         <v>227.39342440000001</v>
       </c>
-      <c r="K50" s="9"/>
-      <c r="L50" s="5">
+      <c r="K50" s="7"/>
+      <c r="L50" s="3">
         <f t="shared" si="7"/>
         <v>53.125467021151898</v>
       </c>
-      <c r="M50" s="5">
+      <c r="M50" s="3">
         <v>61.370740789999999</v>
       </c>
-      <c r="N50" s="5"/>
-      <c r="O50" s="5">
+      <c r="N50" s="3"/>
+      <c r="O50" s="3">
         <v>102.3</v>
       </c>
-      <c r="P50" s="5">
+      <c r="P50" s="3">
         <v>102</v>
       </c>
-      <c r="Q50" s="5">
+      <c r="Q50" s="3">
         <v>101.6</v>
       </c>
-      <c r="R50" s="5">
+      <c r="R50" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S50" s="5">
+      <c r="S50" s="3">
         <v>102.7</v>
       </c>
-      <c r="T50" s="5">
+      <c r="T50" s="3">
         <v>76</v>
       </c>
-      <c r="U50" s="9"/>
-      <c r="V50" s="5">
+      <c r="U50" s="7"/>
+      <c r="V50" s="3">
         <f t="shared" ref="V50:V73" si="8">B50/$I50*100</f>
         <v>77.595781067305666</v>
       </c>
-      <c r="W50" s="5">
+      <c r="W50" s="3">
         <f t="shared" ref="W50:W73" si="9">C50/$I50*100</f>
         <v>2.6775905638852597</v>
       </c>
-      <c r="X50" s="5">
+      <c r="X50" s="3">
         <f t="shared" ref="X50:X73" si="10">D50/$I50*100</f>
         <v>9.7815373043207821</v>
       </c>
-      <c r="Y50" s="5">
+      <c r="Y50" s="3">
         <f t="shared" ref="Y50:Y73" si="11">E50/$I50*100</f>
         <v>6.3489383724000259E-2</v>
       </c>
-      <c r="Z50" s="5">
+      <c r="Z50" s="3">
         <f t="shared" ref="Z50:Z73" si="12">F50/$I50*100</f>
         <v>1.8765006881584983E-2</v>
       </c>
@@ -42236,59 +42230,59 @@
       <c r="H51">
         <v>450</v>
       </c>
-      <c r="I51" s="5">
+      <c r="I51" s="3">
         <f t="shared" si="5"/>
         <v>12202.605561795001</v>
       </c>
-      <c r="J51" s="5">
+      <c r="J51" s="3">
         <f t="shared" si="6"/>
         <v>229.24571610000004</v>
       </c>
-      <c r="K51" s="9"/>
-      <c r="L51" s="5">
+      <c r="K51" s="7"/>
+      <c r="L51" s="3">
         <f t="shared" si="7"/>
         <v>53.229372262171573</v>
       </c>
-      <c r="M51" s="5">
+      <c r="M51" s="3">
         <v>60.067473990000003</v>
       </c>
-      <c r="N51" s="5"/>
-      <c r="O51" s="5">
+      <c r="N51" s="3"/>
+      <c r="O51" s="3">
         <v>102.3</v>
       </c>
-      <c r="P51" s="5">
+      <c r="P51" s="3">
         <v>102</v>
       </c>
-      <c r="Q51" s="5">
+      <c r="Q51" s="3">
         <v>101.6</v>
       </c>
-      <c r="R51" s="5">
+      <c r="R51" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S51" s="5">
+      <c r="S51" s="3">
         <v>102.7</v>
       </c>
-      <c r="T51" s="5">
+      <c r="T51" s="3">
         <v>76</v>
       </c>
-      <c r="U51" s="9"/>
-      <c r="V51" s="5">
+      <c r="U51" s="7"/>
+      <c r="V51" s="3">
         <f t="shared" si="8"/>
         <v>78.180638976555244</v>
       </c>
-      <c r="W51" s="5">
+      <c r="W51" s="3">
         <f t="shared" si="9"/>
         <v>2.6257367057996426</v>
       </c>
-      <c r="X51" s="5">
+      <c r="X51" s="3">
         <f t="shared" si="10"/>
         <v>9.6054702503026892</v>
       </c>
-      <c r="Y51" s="5">
+      <c r="Y51" s="3">
         <f t="shared" si="11"/>
         <v>6.0601702067244391E-2</v>
       </c>
-      <c r="Z51" s="5">
+      <c r="Z51" s="3">
         <f t="shared" si="12"/>
         <v>1.7452295882345401E-2</v>
       </c>
@@ -42336,59 +42330,59 @@
       <c r="H52">
         <v>450</v>
       </c>
-      <c r="I52" s="5">
+      <c r="I52" s="3">
         <f t="shared" si="5"/>
         <v>12385.221646146001</v>
       </c>
-      <c r="J52" s="5">
+      <c r="J52" s="3">
         <f t="shared" si="6"/>
         <v>230.93431240000001</v>
       </c>
-      <c r="K52" s="9"/>
-      <c r="L52" s="5">
+      <c r="K52" s="7"/>
+      <c r="L52" s="3">
         <f t="shared" si="7"/>
         <v>53.630928714887673</v>
       </c>
-      <c r="M52" s="5">
+      <c r="M52" s="3">
         <v>58.791883319999997</v>
       </c>
-      <c r="N52" s="5"/>
-      <c r="O52" s="5">
+      <c r="N52" s="3"/>
+      <c r="O52" s="3">
         <v>102.3</v>
       </c>
-      <c r="P52" s="5">
+      <c r="P52" s="3">
         <v>102</v>
       </c>
-      <c r="Q52" s="5">
+      <c r="Q52" s="3">
         <v>101.6</v>
       </c>
-      <c r="R52" s="5">
+      <c r="R52" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S52" s="5">
+      <c r="S52" s="3">
         <v>102.7</v>
       </c>
-      <c r="T52" s="5">
+      <c r="T52" s="3">
         <v>76</v>
       </c>
-      <c r="U52" s="9"/>
-      <c r="V52" s="5">
+      <c r="U52" s="7"/>
+      <c r="V52" s="3">
         <f t="shared" si="8"/>
         <v>78.608268880109733</v>
       </c>
-      <c r="W52" s="5">
+      <c r="W52" s="3">
         <f t="shared" si="9"/>
         <v>2.5623556103152434</v>
       </c>
-      <c r="X52" s="5">
+      <c r="X52" s="3">
         <f t="shared" si="10"/>
         <v>9.3868989043225639</v>
       </c>
-      <c r="Y52" s="5">
+      <c r="Y52" s="3">
         <f t="shared" si="11"/>
         <v>5.748959151825634E-2</v>
       </c>
-      <c r="Z52" s="5">
+      <c r="Z52" s="3">
         <f t="shared" si="12"/>
         <v>1.6089953574792152E-2</v>
       </c>
@@ -42436,61 +42430,61 @@
       <c r="H53">
         <v>450</v>
       </c>
-      <c r="I53" s="5">
+      <c r="I53" s="3">
         <f t="shared" si="5"/>
         <v>12565.504791508998</v>
       </c>
-      <c r="J53" s="5">
+      <c r="J53" s="3">
         <f t="shared" si="6"/>
         <v>232.48673840000001</v>
       </c>
-      <c r="K53" s="9"/>
-      <c r="L53" s="5">
+      <c r="K53" s="7"/>
+      <c r="L53" s="3">
         <f t="shared" si="7"/>
         <v>54.048264765492526</v>
       </c>
-      <c r="M53" s="5">
+      <c r="M53" s="3">
         <v>57.54338104</v>
       </c>
-      <c r="N53" s="5">
+      <c r="N53" s="3">
         <v>60</v>
       </c>
-      <c r="O53" s="5">
+      <c r="O53" s="3">
         <v>102.3</v>
       </c>
-      <c r="P53" s="5">
+      <c r="P53" s="3">
         <v>102</v>
       </c>
-      <c r="Q53" s="5">
+      <c r="Q53" s="3">
         <v>101.6</v>
       </c>
-      <c r="R53" s="5">
+      <c r="R53" s="3">
         <v>74.400000000000006</v>
       </c>
-      <c r="S53" s="5">
+      <c r="S53" s="3">
         <v>102.7</v>
       </c>
-      <c r="T53" s="5">
+      <c r="T53" s="3">
         <v>76</v>
       </c>
-      <c r="U53" s="9"/>
-      <c r="V53" s="5">
+      <c r="U53" s="7"/>
+      <c r="V53" s="3">
         <f t="shared" si="8"/>
         <v>79.019573807409259</v>
       </c>
-      <c r="W53" s="5">
+      <c r="W53" s="3">
         <f t="shared" si="9"/>
         <v>2.5012807301811204</v>
       </c>
-      <c r="X53" s="5">
+      <c r="X53" s="3">
         <f t="shared" si="10"/>
         <v>9.1763828284810867</v>
       </c>
-      <c r="Y53" s="5">
+      <c r="Y53" s="3">
         <f t="shared" si="11"/>
         <v>5.4478034218137669E-2</v>
       </c>
-      <c r="Z53" s="5">
+      <c r="Z53" s="3">
         <f t="shared" si="12"/>
         <v>1.4773073106099025E-2</v>
       </c>
@@ -42541,55 +42535,55 @@
       <c r="H54">
         <v>450</v>
       </c>
-      <c r="I54" s="5">
+      <c r="I54" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J54" s="5">
+      <c r="J54" s="3">
         <f t="shared" si="6"/>
         <v>233.92404590000001</v>
       </c>
-      <c r="K54" s="9"/>
-      <c r="L54" s="5">
+      <c r="K54" s="7"/>
+      <c r="L54" s="3">
         <f t="shared" si="7"/>
         <v>54.491707614608238</v>
       </c>
-      <c r="M54" s="5">
+      <c r="M54" s="3">
         <v>56.321391920000003</v>
       </c>
-      <c r="N54" s="5"/>
-      <c r="O54" s="5"/>
-      <c r="P54" s="5">
+      <c r="N54" s="3"/>
+      <c r="O54" s="3"/>
+      <c r="P54" s="3">
         <v>102</v>
       </c>
-      <c r="Q54" s="5">
+      <c r="Q54" s="3">
         <v>101.6</v>
       </c>
-      <c r="R54" s="5"/>
-      <c r="S54" s="5">
+      <c r="R54" s="3"/>
+      <c r="S54" s="3">
         <v>102.7</v>
       </c>
-      <c r="T54" s="5">
+      <c r="T54" s="3">
         <v>76</v>
       </c>
-      <c r="U54" s="9"/>
-      <c r="V54" s="5">
+      <c r="U54" s="7"/>
+      <c r="V54" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W54" s="5">
+      <c r="W54" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X54" s="5">
+      <c r="X54" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y54" s="5">
+      <c r="Y54" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z54" s="5">
+      <c r="Z54" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -42637,55 +42631,55 @@
       <c r="H55">
         <v>450</v>
       </c>
-      <c r="I55" s="5">
+      <c r="I55" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J55" s="5">
+      <c r="J55" s="3">
         <f t="shared" si="6"/>
         <v>235.2627057</v>
       </c>
-      <c r="K55" s="9"/>
-      <c r="L55" s="5">
+      <c r="K55" s="7"/>
+      <c r="L55" s="3">
         <f t="shared" si="7"/>
         <v>54.181646322913124</v>
       </c>
-      <c r="M55" s="5">
+      <c r="M55" s="3">
         <v>55.125352909999997</v>
       </c>
-      <c r="N55" s="5"/>
-      <c r="O55" s="5"/>
-      <c r="P55" s="5">
+      <c r="N55" s="3"/>
+      <c r="O55" s="3"/>
+      <c r="P55" s="3">
         <v>102</v>
       </c>
-      <c r="Q55" s="5">
+      <c r="Q55" s="3">
         <v>101.6</v>
       </c>
-      <c r="R55" s="5"/>
-      <c r="S55" s="5">
+      <c r="R55" s="3"/>
+      <c r="S55" s="3">
         <v>102.7</v>
       </c>
-      <c r="T55" s="5">
+      <c r="T55" s="3">
         <v>76</v>
       </c>
-      <c r="U55" s="9"/>
-      <c r="V55" s="5">
+      <c r="U55" s="7"/>
+      <c r="V55" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W55" s="5">
+      <c r="W55" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X55" s="5">
+      <c r="X55" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y55" s="5">
+      <c r="Y55" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z55" s="5">
+      <c r="Z55" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -42733,55 +42727,55 @@
       <c r="H56">
         <v>450</v>
       </c>
-      <c r="I56" s="5">
+      <c r="I56" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J56" s="5">
+      <c r="J56" s="3">
         <f t="shared" si="6"/>
         <v>236.51585300000002</v>
       </c>
-      <c r="K56" s="9"/>
-      <c r="L56" s="5">
+      <c r="K56" s="7"/>
+      <c r="L56" s="3">
         <f t="shared" si="7"/>
         <v>53.894572188397859</v>
       </c>
-      <c r="M56" s="5">
+      <c r="M56" s="3">
         <v>53.95471294</v>
       </c>
-      <c r="N56" s="5"/>
-      <c r="O56" s="5"/>
-      <c r="P56" s="5">
+      <c r="N56" s="3"/>
+      <c r="O56" s="3"/>
+      <c r="P56" s="3">
         <v>102</v>
       </c>
-      <c r="Q56" s="5">
+      <c r="Q56" s="3">
         <v>101.6</v>
       </c>
-      <c r="R56" s="5"/>
-      <c r="S56" s="5">
+      <c r="R56" s="3"/>
+      <c r="S56" s="3">
         <v>102.7</v>
       </c>
-      <c r="T56" s="5">
+      <c r="T56" s="3">
         <v>76</v>
       </c>
-      <c r="U56" s="9"/>
-      <c r="V56" s="5">
+      <c r="U56" s="7"/>
+      <c r="V56" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W56" s="5">
+      <c r="W56" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X56" s="5">
+      <c r="X56" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y56" s="5">
+      <c r="Y56" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z56" s="5">
+      <c r="Z56" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -42829,55 +42823,55 @@
       <c r="H57">
         <v>450</v>
       </c>
-      <c r="I57" s="5">
+      <c r="I57" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J57" s="5">
+      <c r="J57" s="3">
         <f t="shared" si="6"/>
         <v>237.69413579999997</v>
       </c>
-      <c r="K57" s="9"/>
-      <c r="L57" s="5">
+      <c r="K57" s="7"/>
+      <c r="L57" s="3">
         <f t="shared" si="7"/>
         <v>53.627409318732546</v>
       </c>
-      <c r="M57" s="5">
+      <c r="M57" s="3">
         <v>52.808932630000001</v>
       </c>
-      <c r="N57" s="5"/>
-      <c r="O57" s="5"/>
-      <c r="P57" s="5">
+      <c r="N57" s="3"/>
+      <c r="O57" s="3"/>
+      <c r="P57" s="3">
         <v>102</v>
       </c>
-      <c r="Q57" s="5">
+      <c r="Q57" s="3">
         <v>101.6</v>
       </c>
-      <c r="R57" s="5"/>
-      <c r="S57" s="5">
+      <c r="R57" s="3"/>
+      <c r="S57" s="3">
         <v>102.7</v>
       </c>
-      <c r="T57" s="5">
+      <c r="T57" s="3">
         <v>76</v>
       </c>
-      <c r="U57" s="9"/>
-      <c r="V57" s="5">
+      <c r="U57" s="7"/>
+      <c r="V57" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W57" s="5">
+      <c r="W57" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X57" s="5">
+      <c r="X57" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y57" s="5">
+      <c r="Y57" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z57" s="5">
+      <c r="Z57" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -42925,55 +42919,55 @@
       <c r="H58">
         <v>450</v>
       </c>
-      <c r="I58" s="5">
+      <c r="I58" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J58" s="5">
+      <c r="J58" s="3">
         <f t="shared" si="6"/>
         <v>238.80630870000002</v>
       </c>
-      <c r="K58" s="9"/>
-      <c r="L58" s="5">
+      <c r="K58" s="7"/>
+      <c r="L58" s="3">
         <f t="shared" si="7"/>
         <v>53.377654814062275</v>
       </c>
-      <c r="M58" s="5">
+      <c r="M58" s="3">
         <v>51.687484079999997</v>
       </c>
-      <c r="N58" s="5"/>
-      <c r="O58" s="5"/>
-      <c r="P58" s="5">
+      <c r="N58" s="3"/>
+      <c r="O58" s="3"/>
+      <c r="P58" s="3">
         <v>102</v>
       </c>
-      <c r="Q58" s="5">
+      <c r="Q58" s="3">
         <v>101.6</v>
       </c>
-      <c r="R58" s="5"/>
-      <c r="S58" s="5">
+      <c r="R58" s="3"/>
+      <c r="S58" s="3">
         <v>102.7</v>
       </c>
-      <c r="T58" s="5">
+      <c r="T58" s="3">
         <v>76</v>
       </c>
-      <c r="U58" s="9"/>
-      <c r="V58" s="5">
+      <c r="U58" s="7"/>
+      <c r="V58" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W58" s="5">
+      <c r="W58" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X58" s="5">
+      <c r="X58" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y58" s="5">
+      <c r="Y58" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z58" s="5">
+      <c r="Z58" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43024,55 +43018,55 @@
       <c r="H59">
         <v>450</v>
       </c>
-      <c r="I59" s="5">
+      <c r="I59" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J59" s="5">
+      <c r="J59" s="3">
         <f t="shared" si="6"/>
         <v>239.85965880000001</v>
       </c>
-      <c r="K59" s="9"/>
-      <c r="L59" s="5">
+      <c r="K59" s="7"/>
+      <c r="L59" s="3">
         <f t="shared" si="7"/>
         <v>53.14324541684455</v>
       </c>
-      <c r="M59" s="5">
+      <c r="M59" s="3">
         <v>50.589850570000003</v>
       </c>
-      <c r="N59" s="5"/>
-      <c r="O59" s="5"/>
-      <c r="P59" s="5">
+      <c r="N59" s="3"/>
+      <c r="O59" s="3"/>
+      <c r="P59" s="3">
         <v>102</v>
       </c>
-      <c r="Q59" s="5">
+      <c r="Q59" s="3">
         <v>101.6</v>
       </c>
-      <c r="R59" s="5"/>
-      <c r="S59" s="5">
+      <c r="R59" s="3"/>
+      <c r="S59" s="3">
         <v>102.7</v>
       </c>
-      <c r="T59" s="5">
+      <c r="T59" s="3">
         <v>76</v>
       </c>
-      <c r="U59" s="9"/>
-      <c r="V59" s="5">
+      <c r="U59" s="7"/>
+      <c r="V59" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W59" s="5">
+      <c r="W59" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X59" s="5">
+      <c r="X59" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y59" s="5">
+      <c r="Y59" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z59" s="5">
+      <c r="Z59" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43120,55 +43114,55 @@
       <c r="H60">
         <v>450</v>
       </c>
-      <c r="I60" s="5">
+      <c r="I60" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J60" s="5">
+      <c r="J60" s="3">
         <f t="shared" si="6"/>
         <v>240.86031829999999</v>
       </c>
-      <c r="K60" s="9"/>
-      <c r="L60" s="5">
+      <c r="K60" s="7"/>
+      <c r="L60" s="3">
         <f t="shared" si="7"/>
         <v>52.922460632690274</v>
       </c>
-      <c r="M60" s="5">
+      <c r="M60" s="3">
         <v>49.515526360000003</v>
       </c>
-      <c r="N60" s="5"/>
-      <c r="O60" s="5"/>
-      <c r="P60" s="5">
+      <c r="N60" s="3"/>
+      <c r="O60" s="3"/>
+      <c r="P60" s="3">
         <v>102</v>
       </c>
-      <c r="Q60" s="5">
+      <c r="Q60" s="3">
         <v>101.6</v>
       </c>
-      <c r="R60" s="5"/>
-      <c r="S60" s="5">
+      <c r="R60" s="3"/>
+      <c r="S60" s="3">
         <v>102.7</v>
       </c>
-      <c r="T60" s="5">
+      <c r="T60" s="3">
         <v>76</v>
       </c>
-      <c r="U60" s="9"/>
-      <c r="V60" s="5">
+      <c r="U60" s="7"/>
+      <c r="V60" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W60" s="5">
+      <c r="W60" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X60" s="5">
+      <c r="X60" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y60" s="5">
+      <c r="Y60" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z60" s="5">
+      <c r="Z60" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43216,55 +43210,55 @@
       <c r="H61">
         <v>450</v>
       </c>
-      <c r="I61" s="5">
+      <c r="I61" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J61" s="5">
+      <c r="J61" s="3">
         <f t="shared" si="6"/>
         <v>241.81349740000002</v>
       </c>
-      <c r="K61" s="9"/>
-      <c r="L61" s="5">
+      <c r="K61" s="7"/>
+      <c r="L61" s="3">
         <f t="shared" si="7"/>
         <v>52.71385117152272</v>
       </c>
-      <c r="M61" s="5">
+      <c r="M61" s="3">
         <v>48.464016460000003</v>
       </c>
-      <c r="N61" s="5"/>
-      <c r="O61" s="5"/>
-      <c r="P61" s="5">
+      <c r="N61" s="3"/>
+      <c r="O61" s="3"/>
+      <c r="P61" s="3">
         <v>102</v>
       </c>
-      <c r="Q61" s="5">
+      <c r="Q61" s="3">
         <v>101.6</v>
       </c>
-      <c r="R61" s="5"/>
-      <c r="S61" s="5">
+      <c r="R61" s="3"/>
+      <c r="S61" s="3">
         <v>102.7</v>
       </c>
-      <c r="T61" s="5">
+      <c r="T61" s="3">
         <v>76</v>
       </c>
-      <c r="U61" s="9"/>
-      <c r="V61" s="5">
+      <c r="U61" s="7"/>
+      <c r="V61" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W61" s="5">
+      <c r="W61" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X61" s="5">
+      <c r="X61" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y61" s="5">
+      <c r="Y61" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z61" s="5">
+      <c r="Z61" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43312,55 +43306,55 @@
       <c r="H62">
         <v>450</v>
       </c>
-      <c r="I62" s="5">
+      <c r="I62" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J62" s="5">
+      <c r="J62" s="3">
         <f t="shared" si="6"/>
         <v>242.72366120000004</v>
       </c>
-      <c r="K62" s="9"/>
-      <c r="L62" s="5">
+      <c r="K62" s="7"/>
+      <c r="L62" s="3">
         <f t="shared" si="7"/>
         <v>52.516185073138622</v>
       </c>
-      <c r="M62" s="5">
+      <c r="M62" s="3">
         <v>47.43483638</v>
       </c>
-      <c r="N62" s="5"/>
-      <c r="O62" s="5"/>
-      <c r="P62" s="5">
+      <c r="N62" s="3"/>
+      <c r="O62" s="3"/>
+      <c r="P62" s="3">
         <v>102</v>
       </c>
-      <c r="Q62" s="5">
+      <c r="Q62" s="3">
         <v>101.6</v>
       </c>
-      <c r="R62" s="5"/>
-      <c r="S62" s="5">
+      <c r="R62" s="3"/>
+      <c r="S62" s="3">
         <v>102.7</v>
       </c>
-      <c r="T62" s="5">
+      <c r="T62" s="3">
         <v>76</v>
       </c>
-      <c r="U62" s="9"/>
-      <c r="V62" s="5">
+      <c r="U62" s="7"/>
+      <c r="V62" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W62" s="5">
+      <c r="W62" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X62" s="5">
+      <c r="X62" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y62" s="5">
+      <c r="Y62" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z62" s="5">
+      <c r="Z62" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43408,55 +43402,55 @@
       <c r="H63">
         <v>450</v>
       </c>
-      <c r="I63" s="5">
+      <c r="I63" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J63" s="5">
+      <c r="J63" s="3">
         <f t="shared" si="6"/>
         <v>243.59466650000002</v>
       </c>
-      <c r="K63" s="9"/>
-      <c r="L63" s="5">
+      <c r="K63" s="7"/>
+      <c r="L63" s="3">
         <f t="shared" si="7"/>
         <v>52.32840643171059</v>
       </c>
-      <c r="M63" s="5">
+      <c r="M63" s="3">
         <v>46.427511940000002</v>
       </c>
-      <c r="N63" s="5"/>
-      <c r="O63" s="5"/>
-      <c r="P63" s="5">
+      <c r="N63" s="3"/>
+      <c r="O63" s="3"/>
+      <c r="P63" s="3">
         <v>102</v>
       </c>
-      <c r="Q63" s="5">
+      <c r="Q63" s="3">
         <v>101.6</v>
       </c>
-      <c r="R63" s="5"/>
-      <c r="S63" s="5">
+      <c r="R63" s="3"/>
+      <c r="S63" s="3">
         <v>102.7</v>
       </c>
-      <c r="T63" s="5">
+      <c r="T63" s="3">
         <v>76</v>
       </c>
-      <c r="U63" s="9"/>
-      <c r="V63" s="5">
+      <c r="U63" s="7"/>
+      <c r="V63" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W63" s="5">
+      <c r="W63" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X63" s="5">
+      <c r="X63" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y63" s="5">
+      <c r="Y63" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z63" s="5">
+      <c r="Z63" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43507,55 +43501,55 @@
       <c r="H64">
         <v>450</v>
       </c>
-      <c r="I64" s="5">
+      <c r="I64" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J64" s="5">
+      <c r="J64" s="3">
         <f t="shared" si="6"/>
         <v>244.42986730000001</v>
       </c>
-      <c r="K64" s="9"/>
-      <c r="L64" s="5">
+      <c r="K64" s="7"/>
+      <c r="L64" s="3">
         <f t="shared" si="7"/>
         <v>52.149603704379203</v>
       </c>
-      <c r="M64" s="5">
+      <c r="M64" s="3">
         <v>45.441578999999997</v>
       </c>
-      <c r="N64" s="5"/>
-      <c r="O64" s="5"/>
-      <c r="P64" s="5">
+      <c r="N64" s="3"/>
+      <c r="O64" s="3"/>
+      <c r="P64" s="3">
         <v>102</v>
       </c>
-      <c r="Q64" s="5">
+      <c r="Q64" s="3">
         <v>101.6</v>
       </c>
-      <c r="R64" s="5"/>
-      <c r="S64" s="5">
+      <c r="R64" s="3"/>
+      <c r="S64" s="3">
         <v>102.7</v>
       </c>
-      <c r="T64" s="5">
+      <c r="T64" s="3">
         <v>76</v>
       </c>
-      <c r="U64" s="9"/>
-      <c r="V64" s="5">
+      <c r="U64" s="7"/>
+      <c r="V64" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W64" s="5">
+      <c r="W64" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X64" s="5">
+      <c r="X64" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y64" s="5">
+      <c r="Y64" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z64" s="5">
+      <c r="Z64" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43603,55 +43597,55 @@
       <c r="H65">
         <v>450</v>
       </c>
-      <c r="I65" s="5">
+      <c r="I65" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J65" s="5">
+      <c r="J65" s="3">
         <f t="shared" si="6"/>
         <v>245.23219999999998</v>
       </c>
-      <c r="K65" s="9"/>
-      <c r="L65" s="5">
+      <c r="K65" s="7"/>
+      <c r="L65" s="3">
         <f t="shared" si="7"/>
         <v>51.978984461294232</v>
       </c>
-      <c r="M65" s="5">
+      <c r="M65" s="3">
         <v>44.476583300000001</v>
       </c>
-      <c r="N65" s="5"/>
-      <c r="O65" s="5"/>
-      <c r="P65" s="5">
+      <c r="N65" s="3"/>
+      <c r="O65" s="3"/>
+      <c r="P65" s="3">
         <v>102</v>
       </c>
-      <c r="Q65" s="5">
+      <c r="Q65" s="3">
         <v>101.6</v>
       </c>
-      <c r="R65" s="5"/>
-      <c r="S65" s="5">
+      <c r="R65" s="3"/>
+      <c r="S65" s="3">
         <v>102.7</v>
       </c>
-      <c r="T65" s="5">
+      <c r="T65" s="3">
         <v>76</v>
       </c>
-      <c r="U65" s="9"/>
-      <c r="V65" s="5">
+      <c r="U65" s="7"/>
+      <c r="V65" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W65" s="5">
+      <c r="W65" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X65" s="5">
+      <c r="X65" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y65" s="5">
+      <c r="Y65" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z65" s="5">
+      <c r="Z65" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43699,55 +43693,55 @@
       <c r="H66">
         <v>450</v>
       </c>
-      <c r="I66" s="5">
+      <c r="I66" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J66" s="5">
+      <c r="J66" s="3">
         <f t="shared" si="6"/>
         <v>246.00424960000001</v>
       </c>
-      <c r="K66" s="9"/>
-      <c r="L66" s="5">
+      <c r="K66" s="7"/>
+      <c r="L66" s="3">
         <f t="shared" si="7"/>
         <v>51.815855758326691</v>
       </c>
-      <c r="M66" s="5">
+      <c r="M66" s="3">
         <v>43.532080209999997</v>
       </c>
-      <c r="N66" s="5"/>
-      <c r="O66" s="5"/>
-      <c r="P66" s="5">
+      <c r="N66" s="3"/>
+      <c r="O66" s="3"/>
+      <c r="P66" s="3">
         <v>102</v>
       </c>
-      <c r="Q66" s="5">
+      <c r="Q66" s="3">
         <v>101.6</v>
       </c>
-      <c r="R66" s="5"/>
-      <c r="S66" s="5">
+      <c r="R66" s="3"/>
+      <c r="S66" s="3">
         <v>102.7</v>
       </c>
-      <c r="T66" s="5">
+      <c r="T66" s="3">
         <v>76</v>
       </c>
-      <c r="U66" s="9"/>
-      <c r="V66" s="5">
+      <c r="U66" s="7"/>
+      <c r="V66" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W66" s="5">
+      <c r="W66" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X66" s="5">
+      <c r="X66" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y66" s="5">
+      <c r="Y66" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z66" s="5">
+      <c r="Z66" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43795,55 +43789,55 @@
       <c r="H67">
         <v>450</v>
       </c>
-      <c r="I67" s="5">
+      <c r="I67" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J67" s="5">
+      <c r="J67" s="3">
         <f t="shared" si="6"/>
         <v>246.74830409999998</v>
       </c>
-      <c r="K67" s="9"/>
-      <c r="L67" s="5">
+      <c r="K67" s="7"/>
+      <c r="L67" s="3">
         <f t="shared" si="7"/>
         <v>51.659608197521948</v>
       </c>
-      <c r="M67" s="5">
+      <c r="M67" s="3">
         <v>42.60763455</v>
       </c>
-      <c r="N67" s="5"/>
-      <c r="O67" s="5"/>
-      <c r="P67" s="5">
+      <c r="N67" s="3"/>
+      <c r="O67" s="3"/>
+      <c r="P67" s="3">
         <v>102</v>
       </c>
-      <c r="Q67" s="5">
+      <c r="Q67" s="3">
         <v>101.6</v>
       </c>
-      <c r="R67" s="5"/>
-      <c r="S67" s="5">
+      <c r="R67" s="3"/>
+      <c r="S67" s="3">
         <v>102.7</v>
       </c>
-      <c r="T67" s="5">
+      <c r="T67" s="3">
         <v>76</v>
       </c>
-      <c r="U67" s="9"/>
-      <c r="V67" s="5">
+      <c r="U67" s="7"/>
+      <c r="V67" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W67" s="5">
+      <c r="W67" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X67" s="5">
+      <c r="X67" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y67" s="5">
+      <c r="Y67" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z67" s="5">
+      <c r="Z67" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43891,55 +43885,55 @@
       <c r="H68">
         <v>450</v>
       </c>
-      <c r="I68" s="5">
+      <c r="I68" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J68" s="5">
+      <c r="J68" s="3">
         <f t="shared" si="6"/>
         <v>247.46639890000003</v>
       </c>
-      <c r="K68" s="9"/>
-      <c r="L68" s="5">
+      <c r="K68" s="7"/>
+      <c r="L68" s="3">
         <f t="shared" si="7"/>
         <v>51.509703013700729</v>
       </c>
-      <c r="M68" s="5">
+      <c r="M68" s="3">
         <v>41.702820389999999</v>
       </c>
-      <c r="N68" s="5"/>
-      <c r="O68" s="5"/>
-      <c r="P68" s="5">
+      <c r="N68" s="3"/>
+      <c r="O68" s="3"/>
+      <c r="P68" s="3">
         <v>102</v>
       </c>
-      <c r="Q68" s="5">
+      <c r="Q68" s="3">
         <v>101.6</v>
       </c>
-      <c r="R68" s="5"/>
-      <c r="S68" s="5">
+      <c r="R68" s="3"/>
+      <c r="S68" s="3">
         <v>102.7</v>
       </c>
-      <c r="T68" s="5">
+      <c r="T68" s="3">
         <v>76</v>
       </c>
-      <c r="U68" s="9"/>
-      <c r="V68" s="5">
+      <c r="U68" s="7"/>
+      <c r="V68" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W68" s="5">
+      <c r="W68" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X68" s="5">
+      <c r="X68" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y68" s="5">
+      <c r="Y68" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z68" s="5">
+      <c r="Z68" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -43990,55 +43984,55 @@
       <c r="H69">
         <v>450</v>
       </c>
-      <c r="I69" s="5">
+      <c r="I69" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J69" s="5">
+      <c r="J69" s="3">
         <f t="shared" si="6"/>
         <v>248.16035240000002</v>
       </c>
-      <c r="K69" s="9"/>
-      <c r="L69" s="5">
+      <c r="K69" s="7"/>
+      <c r="L69" s="3">
         <f t="shared" si="7"/>
         <v>51.365661718044031</v>
       </c>
-      <c r="M69" s="5">
+      <c r="M69" s="3">
         <v>40.817220829999997</v>
       </c>
-      <c r="N69" s="5"/>
-      <c r="O69" s="5"/>
-      <c r="P69" s="5">
+      <c r="N69" s="3"/>
+      <c r="O69" s="3"/>
+      <c r="P69" s="3">
         <v>102</v>
       </c>
-      <c r="Q69" s="5">
+      <c r="Q69" s="3">
         <v>101.6</v>
       </c>
-      <c r="R69" s="5"/>
-      <c r="S69" s="5">
+      <c r="R69" s="3"/>
+      <c r="S69" s="3">
         <v>102.7</v>
       </c>
-      <c r="T69" s="5">
+      <c r="T69" s="3">
         <v>76</v>
       </c>
-      <c r="U69" s="9"/>
-      <c r="V69" s="5">
+      <c r="U69" s="7"/>
+      <c r="V69" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W69" s="5">
+      <c r="W69" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X69" s="5">
+      <c r="X69" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y69" s="5">
+      <c r="Y69" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z69" s="5">
+      <c r="Z69" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -44086,55 +44080,55 @@
       <c r="H70">
         <v>450</v>
       </c>
-      <c r="I70" s="5">
+      <c r="I70" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J70" s="5">
+      <c r="J70" s="3">
         <f t="shared" si="6"/>
         <v>248.83179619999999</v>
       </c>
-      <c r="K70" s="9"/>
-      <c r="L70" s="5">
+      <c r="K70" s="7"/>
+      <c r="L70" s="3">
         <f t="shared" si="7"/>
         <v>51.227057425424789</v>
       </c>
-      <c r="M70" s="5">
+      <c r="M70" s="3">
         <v>39.950427830000002</v>
       </c>
-      <c r="N70" s="5"/>
-      <c r="O70" s="5"/>
-      <c r="P70" s="5">
+      <c r="N70" s="3"/>
+      <c r="O70" s="3"/>
+      <c r="P70" s="3">
         <v>102</v>
       </c>
-      <c r="Q70" s="5">
+      <c r="Q70" s="3">
         <v>101.6</v>
       </c>
-      <c r="R70" s="5"/>
-      <c r="S70" s="5">
+      <c r="R70" s="3"/>
+      <c r="S70" s="3">
         <v>102.7</v>
       </c>
-      <c r="T70" s="5">
+      <c r="T70" s="3">
         <v>76</v>
       </c>
-      <c r="U70" s="9"/>
-      <c r="V70" s="5">
+      <c r="U70" s="7"/>
+      <c r="V70" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W70" s="5">
+      <c r="W70" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X70" s="5">
+      <c r="X70" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y70" s="5">
+      <c r="Y70" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z70" s="5">
+      <c r="Z70" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -44182,55 +44176,55 @@
       <c r="H71">
         <v>450</v>
       </c>
-      <c r="I71" s="5">
+      <c r="I71" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J71" s="5">
+      <c r="J71" s="3">
         <f t="shared" si="6"/>
         <v>249.4822001</v>
       </c>
-      <c r="K71" s="9"/>
-      <c r="L71" s="5">
+      <c r="K71" s="7"/>
+      <c r="L71" s="3">
         <f t="shared" si="7"/>
         <v>51.093507705558338</v>
       </c>
-      <c r="M71" s="5">
+      <c r="M71" s="3">
         <v>39.102042009999998</v>
       </c>
-      <c r="N71" s="5"/>
-      <c r="O71" s="5"/>
-      <c r="P71" s="5">
+      <c r="N71" s="3"/>
+      <c r="O71" s="3"/>
+      <c r="P71" s="3">
         <v>102</v>
       </c>
-      <c r="Q71" s="5">
+      <c r="Q71" s="3">
         <v>101.6</v>
       </c>
-      <c r="R71" s="5"/>
-      <c r="S71" s="5">
+      <c r="R71" s="3"/>
+      <c r="S71" s="3">
         <v>102.7</v>
       </c>
-      <c r="T71" s="5">
+      <c r="T71" s="3">
         <v>76</v>
       </c>
-      <c r="U71" s="9"/>
-      <c r="V71" s="5">
+      <c r="U71" s="7"/>
+      <c r="V71" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W71" s="5">
+      <c r="W71" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X71" s="5">
+      <c r="X71" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y71" s="5">
+      <c r="Y71" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z71" s="5">
+      <c r="Z71" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -44278,55 +44272,55 @@
       <c r="H72">
         <v>450</v>
       </c>
-      <c r="I72" s="5">
+      <c r="I72" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J72" s="5">
+      <c r="J72" s="3">
         <f t="shared" si="6"/>
         <v>250.11289269999997</v>
       </c>
-      <c r="K72" s="9"/>
-      <c r="L72" s="5">
+      <c r="K72" s="7"/>
+      <c r="L72" s="3">
         <f t="shared" si="7"/>
         <v>50.964668696620926</v>
       </c>
-      <c r="M72" s="5">
+      <c r="M72" s="3">
         <v>38.271672479999999</v>
       </c>
-      <c r="N72" s="5"/>
-      <c r="O72" s="5"/>
-      <c r="P72" s="5">
+      <c r="N72" s="3"/>
+      <c r="O72" s="3"/>
+      <c r="P72" s="3">
         <v>102</v>
       </c>
-      <c r="Q72" s="5">
+      <c r="Q72" s="3">
         <v>101.6</v>
       </c>
-      <c r="R72" s="5"/>
-      <c r="S72" s="5">
+      <c r="R72" s="3"/>
+      <c r="S72" s="3">
         <v>102.7</v>
       </c>
-      <c r="T72" s="5">
+      <c r="T72" s="3">
         <v>76</v>
       </c>
-      <c r="U72" s="9"/>
-      <c r="V72" s="5">
+      <c r="U72" s="7"/>
+      <c r="V72" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W72" s="5">
+      <c r="W72" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X72" s="5">
+      <c r="X72" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y72" s="5">
+      <c r="Y72" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z72" s="5">
+      <c r="Z72" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -44374,57 +44368,57 @@
       <c r="H73">
         <v>450</v>
       </c>
-      <c r="I73" s="5">
+      <c r="I73" s="3">
         <f t="shared" si="5"/>
         <v>12746.920713208998</v>
       </c>
-      <c r="J73" s="5">
+      <c r="J73" s="3">
         <f t="shared" si="6"/>
         <v>250.72507910000002</v>
       </c>
-      <c r="K73" s="9"/>
-      <c r="L73" s="5">
+      <c r="K73" s="7"/>
+      <c r="L73" s="3">
         <f t="shared" si="7"/>
         <v>50.840230099698061</v>
       </c>
-      <c r="M73" s="5">
+      <c r="M73" s="3">
         <v>37.458936649999998</v>
       </c>
-      <c r="N73" s="5">
+      <c r="N73" s="3">
         <v>42</v>
       </c>
-      <c r="O73" s="5"/>
-      <c r="P73" s="5">
+      <c r="O73" s="3"/>
+      <c r="P73" s="3">
         <v>102</v>
       </c>
-      <c r="Q73" s="5">
+      <c r="Q73" s="3">
         <v>101.6</v>
       </c>
-      <c r="R73" s="5"/>
-      <c r="S73" s="5">
+      <c r="R73" s="3"/>
+      <c r="S73" s="3">
         <v>102.7</v>
       </c>
-      <c r="T73" s="5">
+      <c r="T73" s="3">
         <v>76</v>
       </c>
-      <c r="U73" s="9"/>
-      <c r="V73" s="5">
+      <c r="U73" s="7"/>
+      <c r="V73" s="3">
         <f t="shared" si="8"/>
         <v>79.393880511964468</v>
       </c>
-      <c r="W73" s="5">
+      <c r="W73" s="3">
         <f t="shared" si="9"/>
         <v>2.4656821601966037</v>
       </c>
-      <c r="X73" s="5">
+      <c r="X73" s="3">
         <f t="shared" si="10"/>
         <v>8.9710247496481053</v>
       </c>
-      <c r="Y73" s="5">
+      <c r="Y73" s="3">
         <f t="shared" si="11"/>
         <v>5.3702695372588399E-2</v>
       </c>
-      <c r="Z73" s="5">
+      <c r="Z73" s="3">
         <f t="shared" si="12"/>
         <v>1.456282070599527E-2</v>
       </c>
@@ -47461,19 +47455,19 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10" t="s">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -51093,4 +51087,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>